<commit_message>
Publish Bitcoin blog post and rebuild blog index/excel
Re-create the Bitcoin markdown post to refresh its created/updated
timestamps, then regenerate the per-post HTML, blog index, and blog
Excel export so they all reflect the new post and correct sort order.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GfutJRktFeaC1enc17tMMk
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -427,7 +427,7 @@
     <col width="245" customWidth="1" min="9" max="9"/>
     <col width="103" customWidth="1" min="10" max="10"/>
     <col width="13838" customWidth="1" min="11" max="11"/>
-    <col width="14915" customWidth="1" min="12" max="12"/>
+    <col width="15856" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1054,83 +1054,53 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Một số cách hình thành ý tưởng công nghệ</t>
+          <t>Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>mot-so-cach-hinh-thanh-y-tuong-cong-nghe</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
+          <t>cach-ma-content-engine-van-hanh-va-thay-doi-tu-duy-dung-content-management-system-cms</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Quy Hai Ng</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>25-05-2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>13-08-2026</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>- [ ] Từ file excel * [ ] Hải vẫn đồng ý với quan điểm chưa có một phần mềm quản lý hay kế toán nào có thể coi là hơi hẳn hay thoát khỏi sự phụ thuộc vào Excel. Chúng chỉ có thể lợi hại khi hỗ trợ cho Excel hoặc liên kết với Excel theo một...</t>
-        </is>
-      </c>
+          <t>25-05-2026</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>data\blogs\Các cách hình thành ý tưởng.md</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>- [ ] Từ file excel
-    * [ ] Hải vẫn đồng ý với quan điểm chưa có một phần mềm quản lý hay kế toán nào có thể coi là hơi hẳn hay thoát khỏi sự phụ thuộc vào Excel. Chúng chỉ có thể lợi hại khi hỗ trợ cho Excel hoặc liên kết với Excel theo một cách nào đó. 
-- [ ] Từ cách thức giảm các thao tác lặp lại
-- [ ] Từ cải tiến những thứ sẵn có - từ những ý tưởng cũ
-    * [ ] Khác với việc tạo ra một thứ gì đó hoàn toàn mới, cách này chỉ tập trung vào việc liệu anh em có thể làm điều gì đó cũ một cách tốt hơn hay không? Một chiếc xe có thể làm cho nó chạy nhanh hơn hay không? Một chiếc laptop có thể làm cho nó nhỏ gọn lại hay không? Liệu nó có ổn định hơn không? Liệu tuổi thọ của nó có cao hơn hay không? Liệu nó có tiết kiệm điện năng hơn hay không?</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>&lt;ul class="task-list"&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Từ file excel&lt;ul class="task-list"&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Hải vẫn đồng ý với quan điểm chưa có một phần mềm quản lý hay kế toán nào có thể coi là hơi hẳn hay thoát khỏi sự phụ thuộc vào Excel. Chúng chỉ có thể lợi hại khi hỗ trợ cho Excel hoặc liên kết với Excel theo một cách nào đó. &lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Từ cách thức giảm các thao tác lặp lại&lt;/li&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Từ cải tiến những thứ sẵn có - từ những ý tưởng cũ&lt;ul class="task-list"&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Khác với việc tạo ra một thứ gì đó hoàn toàn mới, cách này chỉ tập trung vào việc liệu anh em có thể làm điều gì đó cũ một cách tốt hơn hay không? Một chiếc xe có thể làm cho nó chạy nhanh hơn hay không? Một chiếc laptop có thể làm cho nó nhỏ gọn lại hay không? Liệu nó có ổn định hơn không? Liệu tuổi thọ của nó có cao hơn hay không? Liệu nó có tiết kiệm điện năng hơn hay không?&lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-&lt;/ul&gt;</t>
-        </is>
-      </c>
+          <t>data\blogs\Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS).md</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS)</t>
+          <t>Cách PR bản thân hay nhất là nâng tầm đối thủ</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>cach-ma-content-engine-van-hanh-va-thay-doi-tu-duy-dung-content-management-system-cms</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>cach-pr-ban-than-hay-nhat-la-nang-tam-doi-thu</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -1141,58 +1111,20 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>25-05-2026</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>30-05-2026</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Có 1 kiểu tâm lý khá phổ biến để bản thân mình trở nên an toàn và có giá trị. Đó là bình thường hóa, tầm thường hóa cá nhân hoặc nhóm khác và nói rằng mình không giống họ. Anh em có thể bắt gặp tâm lý này ở bất kỳ đâu. `Học sinh trường chuy...</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>data\blogs\Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS).md</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Cách PR bản thân hay nhất là nâng tầm đối thủ</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>cach-pr-ban-than-hay-nhat-la-nang-tam-doi-thu</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>25-05-2026</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>30-05-2026</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Có 1 kiểu tâm lý khá phổ biến để bản thân mình trở nên an toàn và có giá trị. Đó là bình thường hóa, tầm thường hóa cá nhân hoặc nhóm khác và nói rằng mình không giống họ. Anh em có thể bắt gặp tâm lý này ở bất kỳ đâu. `Học sinh trường chuy...</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
           <t>data\blogs\Cách PR bản thân hay nhất là nâng tầm đối thủ.md</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t># Cách PR bản thân hay nhất là nâng tầm đối thủ
 Có 1 kiểu tâm lý khá phổ biến để bản thân mình trở nên an toàn và có giá trị. Đó là bình thường hóa, tầm thường hóa cá nhân hoặc nhóm khác và nói rằng mình không giống họ. Anh em có thể bắt gặp tâm lý này ở bất kỳ đâu. `Học sinh trường chuyên toàn là gà công nghiệp, không học đều các môn. Giáo sư tiến sĩ Việt Nam toàn là trên giấy. Đại gia Việt chỉ giỏi phân lô bán nền. Công nghệ của Việt Nam toàn là sao chép, thay nhãn. Con nhà giàu mà có sự nghiệp thì cũng chẳng có gì đặc biệt, nền tảng gia đình để lại sẵn rồi, không giàu được nữa thì coi như vứt.`
@@ -1207,7 +1139,7 @@
 # Kết</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>&lt;h1 id="cach-pr-ban-than-hay-nhat-la-nang-tam-oi-thu"&gt;Cách PR bản thân hay nhất là nâng tầm đối thủ&lt;/h1&gt;
 &lt;p&gt;Có 1 kiểu tâm lý khá phổ biến để bản thân mình trở nên an toàn và có giá trị. Đó là bình thường hóa, tầm thường hóa cá nhân hoặc nhóm khác và nói rằng mình không giống họ. Anh em có thể bắt gặp tâm lý này ở bất kỳ đâu. &lt;code&gt;Học sinh trường chuyên toàn là gà công nghiệp, không học đều các môn. Giáo sư tiến sĩ Việt Nam toàn là trên giấy. Đại gia Việt chỉ giỏi phân lô bán nền. Công nghệ của Việt Nam toàn là sao chép, thay nhãn. Con nhà giàu mà có sự nghiệp thì cũng chẳng có gì đặc biệt, nền tảng gia đình để lại sẵn rồi, không giàu được nữa thì coi như vứt.&lt;/code&gt;&lt;/p&gt;
@@ -1223,50 +1155,50 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Giáp kèo môi giới</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>giap-keo-moi-gioi</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>15-07-2026</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ng...</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>data\blogs\Giáp kèo môi giới.md</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t># Giáp kèo môi giới
 Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ngành nghề khác, tạo ra giá trị và tồn tại tới tận ngày nay là vì giải quyết vấn đề cho người khác và có thể tạo ra thu nhập. Từ nông sản, bảo hiểm, tài chính - chứng khoán, gia sư, nhà đất cho tới việc làm hay thậm chí là mai mối. Những ngành nghề đó phát triển mạnh tới tận ngày nay là vì xã hội thực sự cần chúng. 
@@ -1289,7 +1221,7 @@
 Cuối cùng, khi 2 bên đang lệch xa suy nghĩ về sản phẩm dịch vụ và về tiền, đừng cố đưa họ đi đến giao dịch vì ngoài kia cũng còn rất nhiều người khác có khả năng cung cấp giải pháp. Tiếp tục tìm kiếm cho tới khi tìm được thì dừng. Tiếp tục tìm giáo viên cho học viên tới khi tìm được người phù hợp về năng lực và về giá. Tiếp tục tìm công việc cho người thất nghiệp cho tới khi tìm được chỗ phù hợp về JD và lương. Tiếp tục tìm quỹ đầu tư cho start-up cho tới khi họ tìm được nhà đầu tư và kêu gọi đủ vốn. Tiếp tục tìm khách để giải ngân cho tới khi đạt chỉ tiêu. Tiếp tục tìm nhà cho tới khi tìm được căn phù hợp trong khả năng tài chính của khách thì thôi.</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>&lt;h1 id="giap-keo-moi-gioi"&gt;Giáp kèo môi giới&lt;/h1&gt;
 &lt;p&gt;Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ngành nghề khác, tạo ra giá trị và tồn tại tới tận ngày nay là vì giải quyết vấn đề cho người khác và có thể tạo ra thu nhập. Từ nông sản, bảo hiểm, tài chính - chứng khoán, gia sư, nhà đất cho tới việc làm hay thậm chí là mai mối. Những ngành nghề đó phát triển mạnh tới tận ngày nay là vì xã hội thực sự cần chúng. &lt;/p&gt;
@@ -1313,114 +1245,114 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Góc nhìn về Sandbox</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>goc-nhin-ve-sandbox</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>sandbox, thử nghiệm</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>09-07-2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>09-07-2026</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>data\blogs\Góc nhìn về sandbox.md</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t># Góc nhìn về Sandbox
+Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="goc-nhin-ve-sandbox"&gt;Góc nhìn về Sandbox&lt;/h1&gt;
+&lt;p&gt;Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Góc nhìn về Sandbox</t>
+          <t>Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>goc-nhin-ve-sandbox</t>
+          <t>goc-nhin-ve-thanh-cong-va-that-bai-tu-cao-thu-tft-3-mua</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Công nghệ</t>
-        </is>
-      </c>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>sandbox, thử nghiệm</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>09-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>09-07-2026</t>
+          <t>05-08-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
+          <t>Winners &amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại?...</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>data\blogs\Góc nhìn về sandbox.md</t>
+          <t>data\blogs\Góc nhìn về thành công và thất bại của cao thủ TFT ba mùa.md</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
-        <is>
-          <t># Góc nhìn về Sandbox
-Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>&lt;h1 id="goc-nhin-ve-sandbox"&gt;Góc nhìn về Sandbox&lt;/h1&gt;
-&lt;p&gt;Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.&lt;/p&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>goc-nhin-ve-thanh-cong-va-that-bai-tu-cao-thu-tft-3-mua</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>05-08-2026</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Winners &amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại?...</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>data\blogs\Góc nhìn về thành công và thất bại của cao thủ TFT ba mùa.md</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
         <is>
           <t># Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa
 Winners &amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại? Thật khó để tìm công thức chung. Vì nếu có, ai ai cũng đã thành công và chẳng còn ai thất bại. 3 mùa đạt mức rank cao thủ TFT, Hải nhìn thấy điều này rất rõ.
@@ -1457,7 +1389,7 @@
 Nhờ cơ chế reset mỗi mùa, Hải không còn áp lực mình là cao thủ, không còn bám víu lấy sự thành công của mùa trước mà thay vào đó là niềm vui bắt đầu lại từ đầu. Niềm vui cạnh tranh với những người chơi mới. Niềm vui được thỏa sức thử lại, được sáng tạo và được vấp ngã. Nếu có DNA của cao thủ TFT, Hải sẽ quay trở lại mức rank cao thủ vào mùa mới như cách Hải đã làm ở những mùa cũ. Còn không, mức rank của Hải khi kết thúc mùa mới sẽ là mức rank chính thức của Hải. Những người giỏi hơn và nỗ lực hơn Hải ở mùa mới, họ hoàn toàn xứng đáng có mức rank cao hơn Hải.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>&lt;h1 id="goc-nhin-ve-thanh-cong-va-that-bai-tu-cao-thu-tft-3-mua"&gt;Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa&lt;/h1&gt;
 &lt;p&gt;Winners &amp;amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại? Thật khó để tìm công thức chung. Vì nếu có, ai ai cũng đã thành công và chẳng còn ai thất bại. 3 mùa đạt mức rank cao thủ TFT, Hải nhìn thấy điều này rất rõ.&lt;/p&gt;
@@ -1497,50 +1429,50 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>ky-nang-cot-loi-de-thanh-cong---danh-cho-tat-ca-moi-nguoi</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào...</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>data\blogs\Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người.md</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t># Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người
 Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...
@@ -1570,7 +1502,7 @@
 Là một người viết, thành công đối với Hải là thuyết phục được người khác đọc hết bài viết của mình. Vì thế Hải sẵn sàng đón nhận mọi ý kiến, bất kể là khen hay chê. Khi ai đó khen Hải, Hải sẽ kiểu: "Ok, cảm ơn bạn nhé, tầm ngày này tuần sau Hải sẽ lại ra bài mới, nhớ đón đọc nha!". Còn khi ai đó chê bai, Hải sẽ biết rằng : "Được rồi, có điều gì đó cần thay đổi!".</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>&lt;h1 id="ky-nang-cot-loi-e-thanh-cong-danh-cho-tat-ca-moi-nguoi"&gt;Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người&lt;/h1&gt;
 &lt;p&gt;Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...&lt;/p&gt;
@@ -1605,54 +1537,54 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>tam-biet-wordpress---vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
         <is>
           <t>web, tech, wp</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>24-05-2026</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gia...</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>data\blogs\Lựa chọn content engine thay vì hệ thống back-end.md</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t># Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS
 Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.
@@ -1705,7 +1637,7 @@
 Với 1 blogger, thay vì phải duy trì một CMS phức tạp với hàng loạt plugin, tài khoản quản trị, cơ sở dữ liệu và các bản vá bảo mật định kỳ, việc thuần tập trung vào sản xuất nội dung mới là ưu tiền hàng đầu. Toàn bộ quá trình còn lại được tự động hóa thông qua content engine để chuyển đổi cắt văn bản và nhúng vào các tập tin định dạng.</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-biet-wordpress-vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms"&gt;Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS&lt;/h1&gt;
 &lt;p&gt;Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.&lt;/p&gt;
@@ -1759,42 +1691,42 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Markdown_Example</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>markdownexample</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>21-07-2026</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Example paragraph</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>data\blogs\Markdown_Example.md</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t># This is heading 1 for title
 Example paragraph
@@ -1843,7 +1775,7 @@
 [^1]: This is the footnote.</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>&lt;h1 id="this-is-heading-1-for-title"&gt;This is heading 1 for title&lt;/h1&gt;
 &lt;p&gt;Example paragraph&lt;/p&gt;
@@ -1902,50 +1834,50 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Một cách kiếm tiền không mới nhưng luôn mới mẻ</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>22-07-2026</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp....</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>data\blogs\Một cách kiếm tiền không mới nhưng luôn mới mẻ.md</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t># Một cách kiếm tiền không mới nhưng luôn mới mẻ
 Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. [^1]
@@ -1989,7 +1921,7 @@
 [^3]: [Content Engine - Vì sao các cá nhân và doanh nghiệp nên quan tâm?](https://haicogihay.com/blog/content-engine---vi-sao-cac-ca-nhan-va-doanh-nghiep-nen-quan-tam)</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me"&gt;Một cách kiếm tiền không mới nhưng luôn mới mẻ&lt;/h1&gt;
 &lt;p&gt;Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt;&lt;/p&gt;
@@ -2044,6 +1976,64 @@
 &lt;/li&gt;
 &lt;/ol&gt;
 &lt;/div&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Một số nơi chứa ý tưởng mới</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>mot-so-noi-chua-y-tuong-moi</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Quy Hai Ng</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>data\blogs\Một số nơi chứa ý tưởng mới.md</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t># Một số nơi chứa ý tưởng mới
+## Từ file excel
+## Từ ứng dụng nhắn tin
+## Từ những cái cũ
+## Kết</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="mot-so-noi-chua-y-tuong-moi"&gt;Một số nơi chứa ý tưởng mới&lt;/h1&gt;
+&lt;h2 id="tu-file-excel"&gt;Từ file excel&lt;/h2&gt;
+&lt;h2 id="tu-ung-dung-nhan-tin"&gt;Từ ứng dụng nhắn tin&lt;/h2&gt;
+&lt;h2 id="tu-nhung-cai-cu"&gt;Từ những cái cũ&lt;/h2&gt;
+&lt;h2 id="ket"&gt;Kết&lt;/h2&gt;</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4151,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>in-draft</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4177,12 +4167,12 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09-08-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4198,7 +4188,7 @@
       <c r="K42" t="inlineStr">
         <is>
           <t># Tại sao Bitcoin cưa đôi?
-Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, vì vậy mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?
+Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?
 ## Một số câu hỏi sẽ được trả lời trong bài viết
 Để dễ tiếp cận với bài viết cho cả những người mới tìm hiểu về Bitcoin, Hải sẽ liệt kê các câu hỏi thường gặp về Bitcoin trước khi đi sâu vào chúng, đó là: 
 - [ ] Tư duy nào hình thành nên sổ cái phi tập trung?
@@ -4214,12 +4204,12 @@
 - [ ] Làm sao để biết giao dịch có hợp lệ hay không?
 - [ ] Tiền hay số dư của Bitcoin đến từ đâu? 
 ## Làm sao để chuyển tiền
-Trong thế giới vật lý, anh em đơn giản là đưa tiền và ghi nhớ là đã đưa hoặc ghi chép lại. Hoặc có thể chuyển khoản qua ngân hàng để ngân hàng nhớ giùm anh em. Anh em sẽ đăng nhập vào app ngân hàng rồi nhập số tài khoản người nhận rồi chuyển tiền, có thể sẽ phải xác minh OTP hoặc sinh trắc. Tất nhiên, để chuyển tiền, anh em cần đảm bảo mình có đủ số tiền đó. Còn qua Bitcoin thì sao? Ý tưởng cơ bản cũng sẽ giống như chuyển khoản nhưng sẽ có một vài điểm đặc biệt hơn đấy:
+Ở ngoài đời, anh em đơn giản là đưa tiền và ghi nhớ là đã đưa hoặc ghi chép lại. Hoặc có thể chuyển khoản qua ngân hàng để ngân hàng nhớ giùm anh em. Còn qua Bitcoin thì sao? Ý tưởng cơ bản cũng sẽ giống như chuyển khoản nhưng sẽ có một vài điểm đặc biệt hơn vì không có tổ chức trung gian như ngân hàng đứng ra chịu trách nhiệm [^1]:
  - Tất cả mọi người khi làm ví Bitcoin sẽ nhận được 2 cái khóa - khóa cá nhân và khóa công khai
  - Khóa cá nhân chỉ có bản thân mình được biết, nói cách khác là chỉ có người giữ nó mới có thể chuyển tiền. Nếu làm mất khóa cá nhân thì coi như xong, coi như là mất toàn bộ tài sản Bitcoin.
  - Khóa công khai là địa chỉ công khai để nhận tiền và là định danh để mọi người làm chứng rằng 2 bên đã giao dịch.
  - Khi chuyển tiền cho ai đó, anh em sẽ nói với mọi người rằng tôi chuyển tiền tới người đó. Anh em phải sử dụng khóa cá nhân mà chỉ riêng anh em biết để làm điều đó. Còn thứ mà mọi người, bao gồm cả người nhận nhìn thấy được là khóa công khai của người gửi đã chuyển một số tiền tới khóa công khai của người nhận.
- - Khi mọi người trong mạng lưới xác nhận hợp lệ, lập tức trừ tiền số dư của người chuyển và tăng tiền số dư của người nhận.
+ - Khi mọi người trong mạng lưới xác nhận hợp lệ, ghi giao dịch vào sổ và lập tức trừ tiền số dư của người chuyển và tăng tiền số dư của người nhận.
  - Nếu khóa cá nhân bị người khác phát hiện, cách tốt nhất là tạo ví Bitcoin mới và chuyển tiền qua ví đó trước khi bị người khác tẩu tán tài sản.
  Mọi giao dịch trên Bitcoin đều được ghi lại, không những thế là ghi lại ở nhiều cuốn sổ khác nhau của nhiều người và nhất quán với nhau. Đây chính là ý tưởng cốt lõi để giải quyết vấn đề từ đơn giản như đóng tiền nhà, mua sắm, hay thiếu nợ cho tới những thứ lớn hơn như hợp đồng mua bán. Đó là làm sao để tôi biết, anh biết và mọi người biết chúng ta đã giao dịch? 
 - [x] Tư duy nào hình thành nên sổ cái phi tập trung?
@@ -4227,35 +4217,35 @@
 - [ ] Làm sao để biết giao dịch có hợp lệ hay không?
 - [ ] Tiền hay số dư của Bitcoin đến từ đâu? 
 ## Làm sao để biết giao dịch có hợp lệ hay không?
-Nếu là mua bán bình thường ở tạp hóa, khi anh em chỉ cầm theo tờ 100k, anh em chỉ có thể mua hàng tối đa 100k. Những món đồ nào làm hóa đơn vượt 100k, anh em buộc phải trả lại. Nếu mua, anh em phải đưa tiền đó để đổi lấy món đồ. Những món được trả lại là những món không được mua, không tạo ra giao dịch và không trừ tiền. Tương tự với ngân hàng, anh em có thể biết được số dư ngay sau khi chuyển do ngân hàng đã nắm giữ cuốn sổ giao dịch. Nếu anh em không đủ tiền để chuyển khoản, ngân hàng sẽ báo không hợp lệ hoặc không cho chuyển.
-Trong Bitcoin cũng vậy, nếu số dư trong ví không đủ, chắc chắn sẽ không thể thực hiện giao dịch và cũng sẽ chẳng được ai ghi lại giao dịch đó vào sổ. Nhưng có 1 rủi ro có thể xảy ra trong giao dịch là một người lợi dụng trong lúc mọi người chưa ghi chép lại giao dịch trong sổ thực hiện cùng lúc 2 giao dịch - gọi là `double-spending`. Hiểu nôm na là bản thân chỉ có 1 đồng nhưng lại chuyển 1 đồng cho cửa hàng trà sữa để mua ly olong trân châu. Tận dụng lúc mạng lưới chưa cập nhật - cùng lúc chuyển 1 đồng để mua bánh mì. Tất nhiên chỉ có giao dịch được xác minh và ghi vào sổ đầu tiên là hợp lệ. Sau giao dịch đó, người đó không còn đồng nào nữa nên không thể tiếp tục chuyển tiền. Lý do việc này có khả năng xảy ra là vì khi không có 1 hệ thống tập trung, sẽ cần có thời gian để tất cả những người có liên quan đồng thuận giao dịch và ghi vào sổ. Vì thế khi giao dịch đầu tiên chưa được đồng thuận dù hợp lệ, số dư tài khoản chưa được cập nhật và người đó có thể dùng để thực hiện giao dịch khác. Bitcoin giải quyết vấn đề này bằng `Proof-of-Work (PoW)`. Đại loại là giao thợ đào có khả năng tính toán, giải quyết sớm nhất và ghi nhận chúng và loại bỏ các giao dịch gây xung đột, sau đó gửi thông tin giao dịch cho những người khác ghi vào sổ.
+Nếu là mua bán bình thường ở tạp hóa, khi anh em chỉ cầm theo tờ 100k, anh em sẽ mua hàng ở mức tối đa 100k. Những món đồ nào làm hóa đơn vượt 100k, anh em buộc phải trả lại. Những món được trả lại là những món không được mua, không tạo ra giao dịch và không trừ tiền. Tương tự với ngân hàng, anh em có thể biết được số dư ngay sau khi chuyển do ngân hàng đã nắm giữ cuốn sổ giao dịch. Nếu anh em không đủ tiền để chuyển khoản, ngân hàng sẽ báo không hợp lệ hoặc không cho chuyển.
+Trong Bitcoin cũng vậy, nếu số dư không đủ, chắc chắn sẽ không thể thực hiện giao dịch và cũng sẽ chẳng được ai ghi lại giao dịch đó vào sổ. Nhưng có 1 rủi ro có thể xảy ra trong giao dịch là một người lợi dụng trong lúc mọi người chưa ghi chép lại giao dịch trong sổ thực hiện cùng lúc 2 giao dịch - gọi là `double-spending`. Hiểu nôm na là bản thân chỉ có 1 đồng nhưng lại chuyển 1 đồng cho cửa hàng trà sữa để mua ly olong trân châu rồi tận dụng lúc mạng lưới chưa cập nhật - cùng lúc chuyển 1 đồng để mua bánh mì. Lý do việc này có khả năng xảy ra là vì khi không có 1 hệ thống tập trung, sẽ cần có thời gian để tất cả những người có liên quan đồng thuận giao dịch và ghi vào sổ. Vì thế khi giao dịch đầu tiên chưa được đồng thuận dù hợp lệ, số dư tài khoản chưa được cập nhật và người đó có thể dùng để thực hiện giao dịch khác.  Tất nhiên chỉ có 1 giao dịch được xác minh và ghi vào sổ đầu tiên là hợp lệ. Sau giao dịch đó, người đó không còn đồng nào nữa nên không thể tiếp tục chuyển tiền.Bitcoin giải quyết vấn đề này bằng `Proof-of-Work (PoW)`[^2]. Đại loại là giao thợ đào có khả năng tính toán, giải quyết sớm nhất và ghi nhận chúng và loại bỏ các giao dịch gây xung đột, loại bỏ spam rồi sau đó gửi thông tin giao dịch cho những người khác ghi vào sổ.
 ## Tiền hay số dư của Bitcoin đến từ đâu?
 - [x] Tư duy nào hình thành nên sổ cái phi tập trung?
 - [x] Làm sao để chuyển tiền?
 - [x] Làm sao để biết giao dịch có hợp lệ hay không?
 - [ ] Tiền hay số dư của Bitcoin đến từ đâu? 
 Hải đoán đây là phần hay nhất và là phần nhiều người đặt vấn đề và có nhiều câu hỏi nhất: Ai là người đầu tiên sở hữu đồng Bitcoin? Đồng Bitcoin đến từ đâu? Số dư Bitcoin đến từ đâu để mà người ta chuyển qua chuyển lại? Giá trị của nó thực sự là gì? Nó có đang bị bơm thổi quá mức hay không? Và trò chơi này có thể bị gian lận hay không? Cha đẻ của Bitcoin có thể tự ý tạo ra và tự thưởng cho mình lượng tiền vô hạn hay không?
-Trước khi trả lời đồng tiền Bitcoin hay BTC đến từ đâu, hãy thử bắt đầu với câu hỏi: "Đồng tiền thông thường trong lưu thông như VND, USD hay Yên Nhật đến từ đâu? Số dư tài khoản trong ngân hàng khởi nguồn từ đâu để người ta chuyển qua chuyển lại?". Xin mời các chuyên gia kinh tế tài chính, các nhà quản trị trả lời. Có người nói rằng tiền đến từ thế chấp tài sản như đất đai để vay nợ, cũng có người nói rằng tiền do ngân hàng trung ương tạo ra và chịu trách nhiệm kiểm soát cung tiền và lãi suất. Hải không biết nhưng Hải chắc chắn rằng tiền được tạo ra để giải quyết vấn đề trao đổi và phục vụ lưu thông hàng hóa, để thanh toán thầu, trả lương, mua sắm... Dù muốn hay không, dù ít hay nhiều, chúng ta cũng cần phải thừa nhận rằng chúng phụ thuộc vào ý chí của tổ chức chính phủ và tổ chức tài chính
-Vì vậy hãy so sánh Bitcoin với vàng để dễ hình dung. Vàng đến từ đâu? Chúng có sẵn trong tự nhiên, có độ hiếm cao và có giới hạn! Làm sao để có vàng? Phải đi tìm kiếm mỏ vàng, rồi phải đào! Bitcoin cũng tương tự, đó là các khối chưa được khai phá và vì thế một người phải dùng tài nguyên tính toán để đào coin và chúng được giới hạn ở con số 21 triệu. Về cơ bản là người đào coin sẽ thử từng kết quả khả dĩ đến khi nào đúng để xác minh giao dịch. Nó có thể được hiểu là phần thưởng cho người tìm được và đào được. Và điều đặc biệt hơn nữa là việc đào được sẽ được công khai lên chuỗi cho tất cả mọi người xem, xác minh và lưu trữ. Phần thưởng là coin sau đó sẽ chảy thẳng về ví của người đào được. 
+Trước khi trả lời đồng tiền Bitcoin hay BTC đến từ đâu, hãy thử bắt đầu với câu hỏi: "Đồng tiền thông thường trong lưu thông như USD hay Yên Nhật đến từ đâu? Số dư tài khoản trong ngân hàng khởi nguồn từ đâu để người ta chuyển qua chuyển lại?". Xin mời các chuyên gia kinh tế tài chính, các nhà quản trị trả lời. Có người nói rằng tiền đến từ thế chấp tài sản như đất đai để vay nợ, cũng có người nói rằng tiền do ngân hàng trung ương tạo ra và chịu trách nhiệm kiểm soát cung tiền và lãi suất. Hải không biết nhưng Hải chắc chắn rằng tiền được tạo ra để giải quyết vấn đề trao đổi và phục vụ lưu thông hàng hóa, để thanh toán thầu, trả lương, mua sắm... Dù muốn hay không, dù ít hay nhiều, chúng ta cũng cần phải thừa nhận rằng chúng phụ thuộc vào ý chí của tổ chức chính phủ và tổ chức tài chính
+Vì vậy hãy so sánh Bitcoin với vàng để dễ hình dung. Vàng đến từ đâu? Chúng có sẵn trong tự nhiên, có độ hiếm cao và có giới hạn! Làm sao để có vàng? Phải đi tìm kiếm mỏ vàng, rồi phải đào! Bitcoin cũng tương tự, đó là các khối chưa được khai phá và vì thế một người phải dùng tài nguyên tính toán để đào coin và chúng được giới hạn ở con số 21 triệu. Về cơ bản là người đào coin sẽ thử từng kết quả khả dĩ đến khi nào đúng để xác minh giao dịch. Nó có thể được hiểu là phần thưởng cho người tìm được và đào được. Và điều đặc biệt hơn nữa là việc đào được sẽ được ghi nhận công khai lên chuỗi cho tất cả mọi người xem, xác minh và lưu trữ. Sau đó, phần thưởng là coin sẽ chảy thẳng về ví của người đào được. 
 ![Công thức cung tiền của Bitcoin](https://lookingglasseducation.com/wp-content/uploads/2023/05/Formula-Main-1-500x297.png)
-Phần thưởng khi đào được quy đổi ra Bitcoin sẽ có xu hướng giảm như công thức trên. Cứ sau mỗi giai đoạn, phần thưởng khi đào được sẽ bị cưa đôi. Và tổng số Bitcoin sẽ giới hạn ở con số 21 triệu như hàm tính tổng trên.
-Vậy cha đẻ của Bitcoin là Satoshi Nakamoto có biết trước về chỗ chứa các Bitcoin chưa được khai phá hay không? Câu trả lời là ông hoàn toàn không biết, trừ khi ông chọn cách đào như những người khác. Dù ông biết thuật toán, biết cơ chế tạo block, biết kiểm tra PoW, nhưng ông không khác gì những người bình thường khác vì những gì ông biết đều là mã nguồn mở. Cái số mà các thợ đào coin phải tìm nó chưa từng được ai đó đẻ ra. Số đó chỉ có thể đi tìm và dùng để thử sao cho khớp chuỗi lệnh. Hệ thống không hề tạo ra số nonce ngẫu nhiên mà mà tạo ra kết quả băm ngẫu nhiên. 
+Phần thưởng khi đào được quy đổi ra Bitcoin sẽ có xu hướng giảm như công thức trên. Cứ sau mỗi giai đoạn, phần thưởng khi đào được sẽ bị cưa đôi. Cứ sau mỗi chu kỳ, phần thưởng coin dành cho người đào được sẽ giảm đi một nửa. Cha đẻ của Bitcoin làm vậy để đảm bảo rằng tổng số Bitcoin sẽ giới hạn ở con số 21 triệu. [^3]
+Vậy cha đẻ của Bitcoin là Satoshi Nakamoto có biết trước về chỗ chứa các Bitcoin chưa được khai phá hay không? Câu trả lời là ông hoàn toàn không biết, trừ khi ông chọn cách đào như những người khác. Dù ông biết thuật toán, biết cơ chế tạo block, biết kiểm tra PoW, nhưng ông không khác gì những người bình thường khác vì những gì ông biết đều được công khai trên mã nguồn mở. Cái số mà các thợ đào coin phải tìm nó chưa từng được ai đó đẻ ra. Số đó chỉ có thể đi tìm và dùng để thử sai tới khi khớp chuỗi. Hệ thống không hề tạo ra số nonce ngẫu nhiên mà mà tạo ra kết quả băm ngẫu nhiên dể mọi người tìm số nounce phù hợp. Ngay cả khi anh em giỏi đến mức biết được seed random, anh em cũng không thể kiểm soát được nội dung và thời điểm giao dịch trong tương lai, và vì thế, không thể biết được chuỗi tiếp theo và càng không thể biết được số nounce nếu như không thử sai. 
 ## Tương lai công nghệ hay chiêu trò thổi bong bóng?
 Khi chúng ta đã đi qua 4 câu hỏi:
 - [x] Tư duy nào hình thành nên sổ cái phi tập trung?
 - [x] Làm sao để chuyển tiền?
 - [x] Làm sao để biết giao dịch có hợp lệ hay không?
 - [x] Tiền hay số dư của Bitcoin đến từ đâu?
-Giá trị một đồng tăng khủng khiếp,
-bong bóng hay tăng trưởng bền vững
-với mỗi quốc gia anh em đang sinh sống Anh, Úc, Mỹ, Canada, Hàn Quốc, Nhật Bản, Đài Loan, Trung Quốc và cả Việt Nam 
-- cuốn sổ ghi chép giao dịch như thế nào
-- tiền đến từ đâu, tiền được tạo ra từ đâu
-- dòng tiền có minh bạch hay không, có sạch hay không
-- ở đâu ông có 10 tỷ gửi tiết kiệm? 
-- ở đâu ông có tiền mua biệt thự, mua Maybach, mua Porsche? 
-- ai là người có quyền quyết định cung tiền? trong Bitcoin là không ai cả.
-- Bitcoin không được bảo chứng bơi ai cả, nếu tôi làm mất khóa cá nhân thì sao? Vậy nếu như bạn đánh rơi tiền thì sao?
+Chúng ta vẫn sẽ còn rất nhiều câu hỏi về giá trị của Bitcoin. Chúng không thể làm trang sức như vàng, cũng không thể làm chỗ ở hay mặt bằng kinh doanh như đất, cũng không phải là dạng đầu tư cho sản xuất như cổ phiếu, cũng không được chính phủ coi như tiền mặt chính thống. Vậy một thứ không thể cầm nắm, không thể sờ, không thể ngửi như Bitcoin thì có giá trị gì? Tại sao 1 Bitcoin quy đổi ra USD lại có giá trị khủng khiếp như vậy? Nó sẽ tăng hay giảm trong tương lai? Điều này liệu sẽ sụp đổ? 
+Như Hải đã trình bày, bản chất của Bitcoin là ghi nhận giao dịch. Tất cả giao dịch được công nhận đều được lưu trên nhiều hệ thống khác nhau và đồng bộ với nhau nên giá trị của nó là đảm bảo các bên nhớ được giao dịch. Về lượng cung, Bitcoin có giới hạn giống như đất đai và vàng, không ai có thể tạo ra thêm Bitcoin. Và đó là lý do tỷ giá Bitcoin so với đồng tiền của hầu hết quốc gia luôn biến động rất mạnh vì lạm phát của tiền truyền thống và vì nhu cầu sở hữu Bitcoin luôn thay đổi. Và cũng có cả sự đầu cơ và thao túng truyền thông làm giá Bitcoin nhảy lên xuống liên tục nữa. Nhưng về dài hạn, lượng tiền mỗi quốc gia có khuynh hướng phát hành thêm, nhân khẩu có xu hướng tăng, năng suất lao động tăng, hiệu quả sản xuất luôn đi lên do tiến bộ về khoa học và công nghệ. Và dù những thứ trên có tăng bao nhiêu đi chăng nữa thì số lượng Bitcoin vẫn không tăng, nên Bitoin vẫn có khả năng tăng giá như đất đai hay vàng. Và chính vì chúng không nằm cố định một chỗ như đất đai, không phải ký gửi hành lý hay kiểm tra khi đi qua an ninh sân bay như vàng, chúng có giá trị riêng là có thể chảy đến bất kỳ đâu, chuyển tới bất kỳ đâu, không phân biệt người gửi/nhận là ai và cũng không chịu sự ảnh hưởng của bất kỳ tổ chức nào. 
+Vì ai có Bitcoin cũng có thể chuyển Bitcoin cho bất kỳ ai, nên Bitcoin bị nhiều người lo ngại rằng sẽ được dùng cho các giao dịch phạm pháp hoặc là rửa tiền. Nhưng quay lại với bản chất của Bitcoin một lần nữa, nó được sinh ra là để giải quyết bài toán ghi chép lại ai đã giao dịch với ai. Vì thế, mọi giao dịch đều được lưu lại và thống nhất ở nhiều nơi. Dù có thể không biết ai đứng đằng sau ví, mọi người đều có thể biết được giao dịch và phân tích khoanh vùng nếu họ thật sự muốn. Và vì thế, nếu muốn biết Bitcoin là tương lai nhân loại hay trò thổi bong bóng, hãy hỏi điều tương tự với mỗi hệ thống tài chính và tiền tệ từ mỗi quốc gia anh em đã và đang sinh sống câu hỏi tương tự mà anh em đã đặt cho Bitcoin:
+- Tiền đến từ đâu, tiền được tạo ra như thế nào?
+- Ai là người có quyền quyết định cung tiền? Ai là người kiểm soát cung tiền?
+- Giao dịch được ghi lại như thế nào?
+- Dòng tiền có minh bạch hay không, có sạch hay không?
+- Ở đâu bạn có 10 tỷ gửi tiết kiệm? 
+- Từ đâu bạn có tiền mua biệt thự, mua Maybach, mua Porsche? 
+- Nếu bạn làm mất địa chỉ ví cá nhân, bạn mất toàn bộ tài sản Bitcoin, vậy nếu như bạn đánh rơi ví tiền ở ngoài đường thì sao?
 [^1]: [Bitcoin: A Peer-to-Peer Electronic Cash System by Satoshi Nakamoto](https://bitcoin.org/bitcoin.pdf)
 [^2]: [Mining - Bitcoin Wiki](https://en.bitcoin.it/wiki/Mining)
 [^3]: [Controlled supply - Bitcoin Wiki](https://en.bitcoin.it/wiki/Controlled_supply)</t>
@@ -4264,7 +4254,7 @@
       <c r="L42" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-bitcoin-cua-oi"&gt;Tại sao Bitcoin cưa đôi?&lt;/h1&gt;
-&lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, vì vậy mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?&lt;/p&gt;
+&lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?&lt;/p&gt;
 &lt;h2 id="mot-so-cau-hoi-se-uoc-tra-loi-trong-bai-viet"&gt;Một số câu hỏi sẽ được trả lời trong bài viết&lt;/h2&gt;
 &lt;p&gt;Để dễ tiếp cận với bài viết cho cả những người mới tìm hiểu về Bitcoin, Hải sẽ liệt kê các câu hỏi thường gặp về Bitcoin trước khi đi sâu vào chúng, đó là: &lt;/p&gt;
 &lt;ul class="task-list"&gt;
@@ -4284,13 +4274,13 @@
 &lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Tiền hay số dư của Bitcoin đến từ đâu? &lt;/li&gt;
 &lt;/ul&gt;
 &lt;h2 id="lam-sao-e-chuyen-tien"&gt;Làm sao để chuyển tiền&lt;/h2&gt;
-&lt;p&gt;Trong thế giới vật lý, anh em đơn giản là đưa tiền và ghi nhớ là đã đưa hoặc ghi chép lại. Hoặc có thể chuyển khoản qua ngân hàng để ngân hàng nhớ giùm anh em. Anh em sẽ đăng nhập vào app ngân hàng rồi nhập số tài khoản người nhận rồi chuyển tiền, có thể sẽ phải xác minh OTP hoặc sinh trắc. Tất nhiên, để chuyển tiền, anh em cần đảm bảo mình có đủ số tiền đó. Còn qua Bitcoin thì sao? Ý tưởng cơ bản cũng sẽ giống như chuyển khoản nhưng sẽ có một vài điểm đặc biệt hơn đấy:&lt;/p&gt;
+&lt;p&gt;Ở ngoài đời, anh em đơn giản là đưa tiền và ghi nhớ là đã đưa hoặc ghi chép lại. Hoặc có thể chuyển khoản qua ngân hàng để ngân hàng nhớ giùm anh em. Còn qua Bitcoin thì sao? Ý tưởng cơ bản cũng sẽ giống như chuyển khoản nhưng sẽ có một vài điểm đặc biệt hơn vì không có tổ chức trung gian như ngân hàng đứng ra chịu trách nhiệm &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt;:&lt;/p&gt;
 &lt;ul&gt;
 &lt;li&gt;Tất cả mọi người khi làm ví Bitcoin sẽ nhận được 2 cái khóa - khóa cá nhân và khóa công khai&lt;/li&gt;
 &lt;li&gt;Khóa cá nhân chỉ có bản thân mình được biết, nói cách khác là chỉ có người giữ nó mới có thể chuyển tiền. Nếu làm mất khóa cá nhân thì coi như xong, coi như là mất toàn bộ tài sản Bitcoin.&lt;/li&gt;
 &lt;li&gt;Khóa công khai là địa chỉ công khai để nhận tiền và là định danh để mọi người làm chứng rằng 2 bên đã giao dịch.&lt;/li&gt;
 &lt;li&gt;Khi chuyển tiền cho ai đó, anh em sẽ nói với mọi người rằng tôi chuyển tiền tới người đó. Anh em phải sử dụng khóa cá nhân mà chỉ riêng anh em biết để làm điều đó. Còn thứ mà mọi người, bao gồm cả người nhận nhìn thấy được là khóa công khai của người gửi đã chuyển một số tiền tới khóa công khai của người nhận.&lt;/li&gt;
-&lt;li&gt;Khi mọi người trong mạng lưới xác nhận hợp lệ, lập tức trừ tiền số dư của người chuyển và tăng tiền số dư của người nhận.&lt;/li&gt;
+&lt;li&gt;Khi mọi người trong mạng lưới xác nhận hợp lệ, ghi giao dịch vào sổ và lập tức trừ tiền số dư của người chuyển và tăng tiền số dư của người nhận.&lt;/li&gt;
 &lt;li&gt;Nếu khóa cá nhân bị người khác phát hiện, cách tốt nhất là tạo ví Bitcoin mới và chuyển tiền qua ví đó trước khi bị người khác tẩu tán tài sản.&lt;/li&gt;
 &lt;/ul&gt;
 &lt;p&gt;Mọi giao dịch trên Bitcoin đều được ghi lại, không những thế là ghi lại ở nhiều cuốn sổ khác nhau của nhiều người và nhất quán với nhau. Đây chính là ý tưởng cốt lõi để giải quyết vấn đề từ đơn giản như đóng tiền nhà, mua sắm, hay thiếu nợ cho tới những thứ lớn hơn như hợp đồng mua bán. Đó là làm sao để tôi biết, anh biết và mọi người biết chúng ta đã giao dịch? &lt;/p&gt;
@@ -4301,8 +4291,8 @@
 &lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Tiền hay số dư của Bitcoin đến từ đâu? &lt;/li&gt;
 &lt;/ul&gt;
 &lt;h2 id="lam-sao-e-biet-giao-dich-co-hop-le-hay-khong"&gt;Làm sao để biết giao dịch có hợp lệ hay không?&lt;/h2&gt;
-&lt;p&gt;Nếu là mua bán bình thường ở tạp hóa, khi anh em chỉ cầm theo tờ 100k, anh em chỉ có thể mua hàng tối đa 100k. Những món đồ nào làm hóa đơn vượt 100k, anh em buộc phải trả lại. Nếu mua, anh em phải đưa tiền đó để đổi lấy món đồ. Những món được trả lại là những món không được mua, không tạo ra giao dịch và không trừ tiền. Tương tự với ngân hàng, anh em có thể biết được số dư ngay sau khi chuyển do ngân hàng đã nắm giữ cuốn sổ giao dịch. Nếu anh em không đủ tiền để chuyển khoản, ngân hàng sẽ báo không hợp lệ hoặc không cho chuyển.&lt;/p&gt;
-&lt;p&gt;Trong Bitcoin cũng vậy, nếu số dư trong ví không đủ, chắc chắn sẽ không thể thực hiện giao dịch và cũng sẽ chẳng được ai ghi lại giao dịch đó vào sổ. Nhưng có 1 rủi ro có thể xảy ra trong giao dịch là một người lợi dụng trong lúc mọi người chưa ghi chép lại giao dịch trong sổ thực hiện cùng lúc 2 giao dịch - gọi là &lt;code&gt;double-spending&lt;/code&gt;. Hiểu nôm na là bản thân chỉ có 1 đồng nhưng lại chuyển 1 đồng cho cửa hàng trà sữa để mua ly olong trân châu. Tận dụng lúc mạng lưới chưa cập nhật - cùng lúc chuyển 1 đồng để mua bánh mì. Tất nhiên chỉ có giao dịch được xác minh và ghi vào sổ đầu tiên là hợp lệ. Sau giao dịch đó, người đó không còn đồng nào nữa nên không thể tiếp tục chuyển tiền. Lý do việc này có khả năng xảy ra là vì khi không có 1 hệ thống tập trung, sẽ cần có thời gian để tất cả những người có liên quan đồng thuận giao dịch và ghi vào sổ. Vì thế khi giao dịch đầu tiên chưa được đồng thuận dù hợp lệ, số dư tài khoản chưa được cập nhật và người đó có thể dùng để thực hiện giao dịch khác. Bitcoin giải quyết vấn đề này bằng &lt;code&gt;Proof-of-Work (PoW)&lt;/code&gt;. Đại loại là giao thợ đào có khả năng tính toán, giải quyết sớm nhất và ghi nhận chúng và loại bỏ các giao dịch gây xung đột, sau đó gửi thông tin giao dịch cho những người khác ghi vào sổ.&lt;/p&gt;
+&lt;p&gt;Nếu là mua bán bình thường ở tạp hóa, khi anh em chỉ cầm theo tờ 100k, anh em sẽ mua hàng ở mức tối đa 100k. Những món đồ nào làm hóa đơn vượt 100k, anh em buộc phải trả lại. Những món được trả lại là những món không được mua, không tạo ra giao dịch và không trừ tiền. Tương tự với ngân hàng, anh em có thể biết được số dư ngay sau khi chuyển do ngân hàng đã nắm giữ cuốn sổ giao dịch. Nếu anh em không đủ tiền để chuyển khoản, ngân hàng sẽ báo không hợp lệ hoặc không cho chuyển.&lt;/p&gt;
+&lt;p&gt;Trong Bitcoin cũng vậy, nếu số dư không đủ, chắc chắn sẽ không thể thực hiện giao dịch và cũng sẽ chẳng được ai ghi lại giao dịch đó vào sổ. Nhưng có 1 rủi ro có thể xảy ra trong giao dịch là một người lợi dụng trong lúc mọi người chưa ghi chép lại giao dịch trong sổ thực hiện cùng lúc 2 giao dịch - gọi là &lt;code&gt;double-spending&lt;/code&gt;. Hiểu nôm na là bản thân chỉ có 1 đồng nhưng lại chuyển 1 đồng cho cửa hàng trà sữa để mua ly olong trân châu rồi tận dụng lúc mạng lưới chưa cập nhật - cùng lúc chuyển 1 đồng để mua bánh mì. Lý do việc này có khả năng xảy ra là vì khi không có 1 hệ thống tập trung, sẽ cần có thời gian để tất cả những người có liên quan đồng thuận giao dịch và ghi vào sổ. Vì thế khi giao dịch đầu tiên chưa được đồng thuận dù hợp lệ, số dư tài khoản chưa được cập nhật và người đó có thể dùng để thực hiện giao dịch khác.  Tất nhiên chỉ có 1 giao dịch được xác minh và ghi vào sổ đầu tiên là hợp lệ. Sau giao dịch đó, người đó không còn đồng nào nữa nên không thể tiếp tục chuyển tiền.Bitcoin giải quyết vấn đề này bằng &lt;code&gt;Proof-of-Work (PoW)&lt;/code&gt;&lt;sup id="fnref:2"&gt;&lt;a class="footnote-ref" href="#fn:2"&gt;2&lt;/a&gt;&lt;/sup&gt;. Đại loại là giao thợ đào có khả năng tính toán, giải quyết sớm nhất và ghi nhận chúng và loại bỏ các giao dịch gây xung đột, loại bỏ spam rồi sau đó gửi thông tin giao dịch cho những người khác ghi vào sổ.&lt;/p&gt;
 &lt;h2 id="tien-hay-so-du-cua-bitcoin-en-tu-au"&gt;Tiền hay số dư của Bitcoin đến từ đâu?&lt;/h2&gt;
 &lt;ul class="task-list"&gt;
 &lt;li class="task-list-item"&gt;&lt;input type="checkbox" checked/&gt; Tư duy nào hình thành nên sổ cái phi tập trung?&lt;/li&gt;
@@ -4311,29 +4301,27 @@
 &lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Tiền hay số dư của Bitcoin đến từ đâu? &lt;/li&gt;
 &lt;/ul&gt;
 &lt;p&gt;Hải đoán đây là phần hay nhất và là phần nhiều người đặt vấn đề và có nhiều câu hỏi nhất: Ai là người đầu tiên sở hữu đồng Bitcoin? Đồng Bitcoin đến từ đâu? Số dư Bitcoin đến từ đâu để mà người ta chuyển qua chuyển lại? Giá trị của nó thực sự là gì? Nó có đang bị bơm thổi quá mức hay không? Và trò chơi này có thể bị gian lận hay không? Cha đẻ của Bitcoin có thể tự ý tạo ra và tự thưởng cho mình lượng tiền vô hạn hay không?&lt;/p&gt;
-&lt;p&gt;Trước khi trả lời đồng tiền Bitcoin hay BTC đến từ đâu, hãy thử bắt đầu với câu hỏi: "Đồng tiền thông thường trong lưu thông như VND, USD hay Yên Nhật đến từ đâu? Số dư tài khoản trong ngân hàng khởi nguồn từ đâu để người ta chuyển qua chuyển lại?". Xin mời các chuyên gia kinh tế tài chính, các nhà quản trị trả lời. Có người nói rằng tiền đến từ thế chấp tài sản như đất đai để vay nợ, cũng có người nói rằng tiền do ngân hàng trung ương tạo ra và chịu trách nhiệm kiểm soát cung tiền và lãi suất. Hải không biết nhưng Hải chắc chắn rằng tiền được tạo ra để giải quyết vấn đề trao đổi và phục vụ lưu thông hàng hóa, để thanh toán thầu, trả lương, mua sắm... Dù muốn hay không, dù ít hay nhiều, chúng ta cũng cần phải thừa nhận rằng chúng phụ thuộc vào ý chí của tổ chức chính phủ và tổ chức tài chính&lt;/p&gt;
-&lt;p&gt;Vì vậy hãy so sánh Bitcoin với vàng để dễ hình dung. Vàng đến từ đâu? Chúng có sẵn trong tự nhiên, có độ hiếm cao và có giới hạn! Làm sao để có vàng? Phải đi tìm kiếm mỏ vàng, rồi phải đào! Bitcoin cũng tương tự, đó là các khối chưa được khai phá và vì thế một người phải dùng tài nguyên tính toán để đào coin và chúng được giới hạn ở con số 21 triệu. Về cơ bản là người đào coin sẽ thử từng kết quả khả dĩ đến khi nào đúng để xác minh giao dịch. Nó có thể được hiểu là phần thưởng cho người tìm được và đào được. Và điều đặc biệt hơn nữa là việc đào được sẽ được công khai lên chuỗi cho tất cả mọi người xem, xác minh và lưu trữ. Phần thưởng là coin sau đó sẽ chảy thẳng về ví của người đào được. &lt;/p&gt;
+&lt;p&gt;Trước khi trả lời đồng tiền Bitcoin hay BTC đến từ đâu, hãy thử bắt đầu với câu hỏi: "Đồng tiền thông thường trong lưu thông như USD hay Yên Nhật đến từ đâu? Số dư tài khoản trong ngân hàng khởi nguồn từ đâu để người ta chuyển qua chuyển lại?". Xin mời các chuyên gia kinh tế tài chính, các nhà quản trị trả lời. Có người nói rằng tiền đến từ thế chấp tài sản như đất đai để vay nợ, cũng có người nói rằng tiền do ngân hàng trung ương tạo ra và chịu trách nhiệm kiểm soát cung tiền và lãi suất. Hải không biết nhưng Hải chắc chắn rằng tiền được tạo ra để giải quyết vấn đề trao đổi và phục vụ lưu thông hàng hóa, để thanh toán thầu, trả lương, mua sắm... Dù muốn hay không, dù ít hay nhiều, chúng ta cũng cần phải thừa nhận rằng chúng phụ thuộc vào ý chí của tổ chức chính phủ và tổ chức tài chính&lt;/p&gt;
+&lt;p&gt;Vì vậy hãy so sánh Bitcoin với vàng để dễ hình dung. Vàng đến từ đâu? Chúng có sẵn trong tự nhiên, có độ hiếm cao và có giới hạn! Làm sao để có vàng? Phải đi tìm kiếm mỏ vàng, rồi phải đào! Bitcoin cũng tương tự, đó là các khối chưa được khai phá và vì thế một người phải dùng tài nguyên tính toán để đào coin và chúng được giới hạn ở con số 21 triệu. Về cơ bản là người đào coin sẽ thử từng kết quả khả dĩ đến khi nào đúng để xác minh giao dịch. Nó có thể được hiểu là phần thưởng cho người tìm được và đào được. Và điều đặc biệt hơn nữa là việc đào được sẽ được ghi nhận công khai lên chuỗi cho tất cả mọi người xem, xác minh và lưu trữ. Sau đó, phần thưởng là coin sẽ chảy thẳng về ví của người đào được. &lt;/p&gt;
 &lt;p&gt;&lt;img alt="Công thức cung tiền của Bitcoin" src="https://lookingglasseducation.com/wp-content/uploads/2023/05/Formula-Main-1-500x297.png" /&gt;&lt;/p&gt;
-&lt;p&gt;Phần thưởng khi đào được quy đổi ra Bitcoin sẽ có xu hướng giảm như công thức trên. Cứ sau mỗi giai đoạn, phần thưởng khi đào được sẽ bị cưa đôi. Và tổng số Bitcoin sẽ giới hạn ở con số 21 triệu như hàm tính tổng trên.&lt;/p&gt;
-&lt;p&gt;Vậy cha đẻ của Bitcoin là Satoshi Nakamoto có biết trước về chỗ chứa các Bitcoin chưa được khai phá hay không? Câu trả lời là ông hoàn toàn không biết, trừ khi ông chọn cách đào như những người khác. Dù ông biết thuật toán, biết cơ chế tạo block, biết kiểm tra PoW, nhưng ông không khác gì những người bình thường khác vì những gì ông biết đều là mã nguồn mở. Cái số mà các thợ đào coin phải tìm nó chưa từng được ai đó đẻ ra. Số đó chỉ có thể đi tìm và dùng để thử sao cho khớp chuỗi lệnh. Hệ thống không hề tạo ra số nonce ngẫu nhiên mà mà tạo ra kết quả băm ngẫu nhiên. &lt;/p&gt;
+&lt;p&gt;Phần thưởng khi đào được quy đổi ra Bitcoin sẽ có xu hướng giảm như công thức trên. Cứ sau mỗi giai đoạn, phần thưởng khi đào được sẽ bị cưa đôi. Cứ sau mỗi chu kỳ, phần thưởng coin dành cho người đào được sẽ giảm đi một nửa. Cha đẻ của Bitcoin làm vậy để đảm bảo rằng tổng số Bitcoin sẽ giới hạn ở con số 21 triệu. &lt;sup id="fnref:3"&gt;&lt;a class="footnote-ref" href="#fn:3"&gt;3&lt;/a&gt;&lt;/sup&gt;&lt;/p&gt;
+&lt;p&gt;Vậy cha đẻ của Bitcoin là Satoshi Nakamoto có biết trước về chỗ chứa các Bitcoin chưa được khai phá hay không? Câu trả lời là ông hoàn toàn không biết, trừ khi ông chọn cách đào như những người khác. Dù ông biết thuật toán, biết cơ chế tạo block, biết kiểm tra PoW, nhưng ông không khác gì những người bình thường khác vì những gì ông biết đều được công khai trên mã nguồn mở. Cái số mà các thợ đào coin phải tìm nó chưa từng được ai đó đẻ ra. Số đó chỉ có thể đi tìm và dùng để thử sai tới khi khớp chuỗi. Hệ thống không hề tạo ra số nonce ngẫu nhiên mà mà tạo ra kết quả băm ngẫu nhiên dể mọi người tìm số nounce phù hợp. Ngay cả khi anh em giỏi đến mức biết được seed random, anh em cũng không thể kiểm soát được nội dung và thời điểm giao dịch trong tương lai, và vì thế, không thể biết được chuỗi tiếp theo và càng không thể biết được số nounce nếu như không thử sai. &lt;/p&gt;
 &lt;h2 id="tuong-lai-cong-nghe-hay-chieu-tro-thoi-bong-bong"&gt;Tương lai công nghệ hay chiêu trò thổi bong bóng?&lt;/h2&gt;
 &lt;p&gt;Khi chúng ta đã đi qua 4 câu hỏi:
 - [x] Tư duy nào hình thành nên sổ cái phi tập trung?
 - [x] Làm sao để chuyển tiền?
 - [x] Làm sao để biết giao dịch có hợp lệ hay không?
 - [x] Tiền hay số dư của Bitcoin đến từ đâu?&lt;/p&gt;
-&lt;p&gt;Giá trị một đồng tăng khủng khiếp,
-bong bóng hay tăng trưởng bền vững&lt;/p&gt;
-&lt;p&gt;với mỗi quốc gia anh em đang sinh sống Anh, Úc, Mỹ, Canada, Hàn Quốc, Nhật Bản, Đài Loan, Trung Quốc và cả Việt Nam &lt;/p&gt;
-&lt;ul&gt;
-&lt;li&gt;cuốn sổ ghi chép giao dịch như thế nào&lt;/li&gt;
-&lt;li&gt;tiền đến từ đâu, tiền được tạo ra từ đâu&lt;/li&gt;
-&lt;li&gt;dòng tiền có minh bạch hay không, có sạch hay không&lt;/li&gt;
-&lt;li&gt;ở đâu ông có 10 tỷ gửi tiết kiệm? &lt;/li&gt;
-&lt;li&gt;ở đâu ông có tiền mua biệt thự, mua Maybach, mua Porsche? &lt;/li&gt;
-&lt;li&gt;ai là người có quyền quyết định cung tiền? trong Bitcoin là không ai cả.&lt;/li&gt;
-&lt;li&gt;Bitcoin không được bảo chứng bơi ai cả, nếu tôi làm mất khóa cá nhân thì sao? Vậy nếu như bạn đánh rơi tiền thì sao?&lt;/li&gt;
-&lt;/ul&gt;
+&lt;p&gt;Chúng ta vẫn sẽ còn rất nhiều câu hỏi về giá trị của Bitcoin. Chúng không thể làm trang sức như vàng, cũng không thể làm chỗ ở hay mặt bằng kinh doanh như đất, cũng không phải là dạng đầu tư cho sản xuất như cổ phiếu, cũng không được chính phủ coi như tiền mặt chính thống. Vậy một thứ không thể cầm nắm, không thể sờ, không thể ngửi như Bitcoin thì có giá trị gì? Tại sao 1 Bitcoin quy đổi ra USD lại có giá trị khủng khiếp như vậy? Nó sẽ tăng hay giảm trong tương lai? Điều này liệu sẽ sụp đổ? &lt;/p&gt;
+&lt;p&gt;Như Hải đã trình bày, bản chất của Bitcoin là ghi nhận giao dịch. Tất cả giao dịch được công nhận đều được lưu trên nhiều hệ thống khác nhau và đồng bộ với nhau nên giá trị của nó là đảm bảo các bên nhớ được giao dịch. Về lượng cung, Bitcoin có giới hạn giống như đất đai và vàng, không ai có thể tạo ra thêm Bitcoin. Và đó là lý do tỷ giá Bitcoin so với đồng tiền của hầu hết quốc gia luôn biến động rất mạnh vì lạm phát của tiền truyền thống và vì nhu cầu sở hữu Bitcoin luôn thay đổi. Và cũng có cả sự đầu cơ và thao túng truyền thông làm giá Bitcoin nhảy lên xuống liên tục nữa. Nhưng về dài hạn, lượng tiền mỗi quốc gia có khuynh hướng phát hành thêm, nhân khẩu có xu hướng tăng, năng suất lao động tăng, hiệu quả sản xuất luôn đi lên do tiến bộ về khoa học và công nghệ. Và dù những thứ trên có tăng bao nhiêu đi chăng nữa thì số lượng Bitcoin vẫn không tăng, nên Bitoin vẫn có khả năng tăng giá như đất đai hay vàng. Và chính vì chúng không nằm cố định một chỗ như đất đai, không phải ký gửi hành lý hay kiểm tra khi đi qua an ninh sân bay như vàng, chúng có giá trị riêng là có thể chảy đến bất kỳ đâu, chuyển tới bất kỳ đâu, không phân biệt người gửi/nhận là ai và cũng không chịu sự ảnh hưởng của bất kỳ tổ chức nào. &lt;/p&gt;
+&lt;p&gt;Vì ai có Bitcoin cũng có thể chuyển Bitcoin cho bất kỳ ai, nên Bitcoin bị nhiều người lo ngại rằng sẽ được dùng cho các giao dịch phạm pháp hoặc là rửa tiền. Nhưng quay lại với bản chất của Bitcoin một lần nữa, nó được sinh ra là để giải quyết bài toán ghi chép lại ai đã giao dịch với ai. Vì thế, mọi giao dịch đều được lưu lại và thống nhất ở nhiều nơi. Dù có thể không biết ai đứng đằng sau ví, mọi người đều có thể biết được giao dịch và phân tích khoanh vùng nếu họ thật sự muốn. Và vì thế, nếu muốn biết Bitcoin là tương lai nhân loại hay trò thổi bong bóng, hãy hỏi điều tương tự với mỗi hệ thống tài chính và tiền tệ từ mỗi quốc gia anh em đã và đang sinh sống câu hỏi tương tự mà anh em đã đặt cho Bitcoin:
+- Tiền đến từ đâu, tiền được tạo ra như thế nào?
+- Ai là người có quyền quyết định cung tiền? Ai là người kiểm soát cung tiền?
+- Giao dịch được ghi lại như thế nào?
+- Dòng tiền có minh bạch hay không, có sạch hay không?
+- Ở đâu bạn có 10 tỷ gửi tiết kiệm? 
+- Từ đâu bạn có tiền mua biệt thự, mua Maybach, mua Porsche? 
+- Nếu bạn làm mất địa chỉ ví cá nhân, bạn mất toàn bộ tài sản Bitcoin, vậy nếu như bạn đánh rơi ví tiền ở ngoài đường thì sao?&lt;/p&gt;
 &lt;div class="footnote"&gt;
 &lt;hr /&gt;
 &lt;ol&gt;

</xml_diff>

<commit_message>
Edit Bitcoin blog post
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="91" customWidth="1" min="1" max="1"/>
@@ -427,7 +427,7 @@
     <col width="245" customWidth="1" min="9" max="9"/>
     <col width="103" customWidth="1" min="10" max="10"/>
     <col width="13838" customWidth="1" min="11" max="11"/>
-    <col width="15856" customWidth="1" min="12" max="12"/>
+    <col width="16121" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1158,17 +1158,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Giáp kèo môi giới</t>
+          <t>Giá trị thặng dư</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>giap-keo-moi-gioi</t>
+          <t>gia-tri-thang-du</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>in-draft</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -1180,25 +1180,75 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>data\blogs\Giá trị thặng dư.md</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t># Giá trị thặng dư</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="gia-tri-thang-du"&gt;Giá trị thặng dư&lt;/h1&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Giáp kèo môi giới</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>giap-keo-moi-gioi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>15-07-2026</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ng...</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>data\blogs\Giáp kèo môi giới.md</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t># Giáp kèo môi giới
 Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ngành nghề khác, tạo ra giá trị và tồn tại tới tận ngày nay là vì giải quyết vấn đề cho người khác và có thể tạo ra thu nhập. Từ nông sản, bảo hiểm, tài chính - chứng khoán, gia sư, nhà đất cho tới việc làm hay thậm chí là mai mối. Những ngành nghề đó phát triển mạnh tới tận ngày nay là vì xã hội thực sự cần chúng. 
@@ -1221,7 +1271,7 @@
 Cuối cùng, khi 2 bên đang lệch xa suy nghĩ về sản phẩm dịch vụ và về tiền, đừng cố đưa họ đi đến giao dịch vì ngoài kia cũng còn rất nhiều người khác có khả năng cung cấp giải pháp. Tiếp tục tìm kiếm cho tới khi tìm được thì dừng. Tiếp tục tìm giáo viên cho học viên tới khi tìm được người phù hợp về năng lực và về giá. Tiếp tục tìm công việc cho người thất nghiệp cho tới khi tìm được chỗ phù hợp về JD và lương. Tiếp tục tìm quỹ đầu tư cho start-up cho tới khi họ tìm được nhà đầu tư và kêu gọi đủ vốn. Tiếp tục tìm khách để giải ngân cho tới khi đạt chỉ tiêu. Tiếp tục tìm nhà cho tới khi tìm được căn phù hợp trong khả năng tài chính của khách thì thôi.</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>&lt;h1 id="giap-keo-moi-gioi"&gt;Giáp kèo môi giới&lt;/h1&gt;
 &lt;p&gt;Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ngành nghề khác, tạo ra giá trị và tồn tại tới tận ngày nay là vì giải quyết vấn đề cho người khác và có thể tạo ra thu nhập. Từ nông sản, bảo hiểm, tài chính - chứng khoán, gia sư, nhà đất cho tới việc làm hay thậm chí là mai mối. Những ngành nghề đó phát triển mạnh tới tận ngày nay là vì xã hội thực sự cần chúng. &lt;/p&gt;
@@ -1245,114 +1295,114 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Góc nhìn về Sandbox</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>goc-nhin-ve-sandbox</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>sandbox, thử nghiệm</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>data\blogs\Góc nhìn về sandbox.md</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t># Góc nhìn về Sandbox
 Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>&lt;h1 id="goc-nhin-ve-sandbox"&gt;Góc nhìn về Sandbox&lt;/h1&gt;
 &lt;p&gt;Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.&lt;/p&gt;</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>goc-nhin-ve-thanh-cong-va-that-bai-tu-cao-thu-tft-3-mua</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>05-08-2026</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Winners &amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại?...</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>data\blogs\Góc nhìn về thành công và thất bại của cao thủ TFT ba mùa.md</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t># Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa
 Winners &amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại? Thật khó để tìm công thức chung. Vì nếu có, ai ai cũng đã thành công và chẳng còn ai thất bại. 3 mùa đạt mức rank cao thủ TFT, Hải nhìn thấy điều này rất rõ.
@@ -1389,7 +1439,7 @@
 Nhờ cơ chế reset mỗi mùa, Hải không còn áp lực mình là cao thủ, không còn bám víu lấy sự thành công của mùa trước mà thay vào đó là niềm vui bắt đầu lại từ đầu. Niềm vui cạnh tranh với những người chơi mới. Niềm vui được thỏa sức thử lại, được sáng tạo và được vấp ngã. Nếu có DNA của cao thủ TFT, Hải sẽ quay trở lại mức rank cao thủ vào mùa mới như cách Hải đã làm ở những mùa cũ. Còn không, mức rank của Hải khi kết thúc mùa mới sẽ là mức rank chính thức của Hải. Những người giỏi hơn và nỗ lực hơn Hải ở mùa mới, họ hoàn toàn xứng đáng có mức rank cao hơn Hải.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>&lt;h1 id="goc-nhin-ve-thanh-cong-va-that-bai-tu-cao-thu-tft-3-mua"&gt;Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa&lt;/h1&gt;
 &lt;p&gt;Winners &amp;amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại? Thật khó để tìm công thức chung. Vì nếu có, ai ai cũng đã thành công và chẳng còn ai thất bại. 3 mùa đạt mức rank cao thủ TFT, Hải nhìn thấy điều này rất rõ.&lt;/p&gt;
@@ -1429,50 +1479,50 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>ky-nang-cot-loi-de-thanh-cong---danh-cho-tat-ca-moi-nguoi</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào...</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>data\blogs\Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người.md</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t># Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người
 Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...
@@ -1502,7 +1552,7 @@
 Là một người viết, thành công đối với Hải là thuyết phục được người khác đọc hết bài viết của mình. Vì thế Hải sẵn sàng đón nhận mọi ý kiến, bất kể là khen hay chê. Khi ai đó khen Hải, Hải sẽ kiểu: "Ok, cảm ơn bạn nhé, tầm ngày này tuần sau Hải sẽ lại ra bài mới, nhớ đón đọc nha!". Còn khi ai đó chê bai, Hải sẽ biết rằng : "Được rồi, có điều gì đó cần thay đổi!".</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>&lt;h1 id="ky-nang-cot-loi-e-thanh-cong-danh-cho-tat-ca-moi-nguoi"&gt;Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người&lt;/h1&gt;
 &lt;p&gt;Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...&lt;/p&gt;
@@ -1537,54 +1587,54 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>tam-biet-wordpress---vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
         <is>
           <t>web, tech, wp</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>24-05-2026</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gia...</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>data\blogs\Lựa chọn content engine thay vì hệ thống back-end.md</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t># Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS
 Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.
@@ -1637,7 +1687,7 @@
 Với 1 blogger, thay vì phải duy trì một CMS phức tạp với hàng loạt plugin, tài khoản quản trị, cơ sở dữ liệu và các bản vá bảo mật định kỳ, việc thuần tập trung vào sản xuất nội dung mới là ưu tiền hàng đầu. Toàn bộ quá trình còn lại được tự động hóa thông qua content engine để chuyển đổi cắt văn bản và nhúng vào các tập tin định dạng.</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-biet-wordpress-vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms"&gt;Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS&lt;/h1&gt;
 &lt;p&gt;Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.&lt;/p&gt;
@@ -1691,42 +1741,42 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Markdown_Example</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>markdownexample</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>21-07-2026</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Example paragraph</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>data\blogs\Markdown_Example.md</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t># This is heading 1 for title
 Example paragraph
@@ -1775,7 +1825,7 @@
 [^1]: This is the footnote.</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>&lt;h1 id="this-is-heading-1-for-title"&gt;This is heading 1 for title&lt;/h1&gt;
 &lt;p&gt;Example paragraph&lt;/p&gt;
@@ -1834,50 +1884,50 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Một cách kiếm tiền không mới nhưng luôn mới mẻ</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>22-07-2026</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp....</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>data\blogs\Một cách kiếm tiền không mới nhưng luôn mới mẻ.md</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t># Một cách kiếm tiền không mới nhưng luôn mới mẻ
 Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. [^1]
@@ -1921,7 +1971,7 @@
 [^3]: [Content Engine - Vì sao các cá nhân và doanh nghiệp nên quan tâm?](https://haicogihay.com/blog/content-engine---vi-sao-cac-ca-nhan-va-doanh-nghiep-nen-quan-tam)</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me"&gt;Một cách kiếm tiền không mới nhưng luôn mới mẻ&lt;/h1&gt;
 &lt;p&gt;Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt;&lt;/p&gt;
@@ -1979,116 +2029,130 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Một số nơi chứa ý tưởng mới</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>mot-so-noi-chua-y-tuong-moi</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Quy Hai Ng</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>17-08-2026</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>- [ ] Excel luôn là nơi - [ ] Hải vẫn đồng ý với quan điểm rằng chưa có phần mềm hay hệ thống nào có thể thay thế hoàn toàn Excel. - [ ] Nếu chúng hỗ trợ cho Excel</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>data\blogs\Một số nơi chứa ý tưởng mới.md</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t># Một số nơi chứa ý tưởng mới
+      <c r="K17" t="inlineStr">
+        <is>
+          <t># Một số nơi chứa ý tưởng mớ
 ## Từ file excel
+- [ ] Excel luôn là nơi
+- [ ] Hải vẫn đồng ý với quan điểm rằng chưa có phần mềm hay hệ thống nào có thể thay thế hoàn toàn Excel.
+- [ ] Nếu chúng hỗ trợ cho Excel
 ## Từ ứng dụng nhắn tin
+Về cơ bản, những gì bạn viết trên các ứng dụng nhắn tin sẽ định hình con người bạn như ngoài đời. 
 ## Từ những cái cũ
 ## Kết</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>&lt;h1 id="mot-so-noi-chua-y-tuong-moi"&gt;Một số nơi chứa ý tưởng mới&lt;/h1&gt;
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="mot-so-noi-chua-y-tuong-mo"&gt;Một số nơi chứa ý tưởng mớ&lt;/h1&gt;
 &lt;h2 id="tu-file-excel"&gt;Từ file excel&lt;/h2&gt;
+&lt;ul class="task-list"&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Excel luôn là nơi&lt;/li&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Hải vẫn đồng ý với quan điểm rằng chưa có phần mềm hay hệ thống nào có thể thay thế hoàn toàn Excel.&lt;/li&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Nếu chúng hỗ trợ cho Excel&lt;/li&gt;
+&lt;/ul&gt;
 &lt;h2 id="tu-ung-dung-nhan-tin"&gt;Từ ứng dụng nhắn tin&lt;/h2&gt;
+&lt;p&gt;Về cơ bản, những gì bạn viết trên các ứng dụng nhắn tin sẽ định hình con người bạn như ngoài đời. &lt;/p&gt;
 &lt;h2 id="tu-nhung-cai-cu"&gt;Từ những cái cũ&lt;/h2&gt;
 &lt;h2 id="ket"&gt;Kết&lt;/h2&gt;</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Một vài góc nhìn nhìn từ thí ngiệm "Vũ trụ 25"</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>mot-vai-goc-nhin-nhin-tu-thi-ngiem-vu-tru-25</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>universe25, tâm lý, thiên đường của loài chuột</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi m...</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>data\blogs\Một vài góc nhìn từ thí nghiệm vũ trụ 25.md</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t># Một vài góc nhìn từ thí nghiệm "Vũ trụ 25"
 Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi mãi hay không?  [^1] Ông chọn ra 4 cặp chuột khỏe mạnh đã được sàng lọc kỹ càng về sức khỏe. Sau đó, đưa chúng vào môi trường 3m x 4.3m, chia thành 16 tháp, tạo được thành 256 hộp tổ, mỗi hộp có sức chứa đủ cho 15 chuột cùng ở - thiên đường đủ để chứa 4000 con chuột. Thức ăn, nước đều được cung cấp đầy đủ, nhiệt độ môi trường được kiểm soát, chất thải của chúng cũng được dọn dẹp, và hoàn toàn không có thú săn mồi. 
@@ -2129,7 +2193,7 @@
 [^4]: [Sáng Thế Ký 3 - Người Nam và Người Nữ Phạm Tội](https://www.bible.com/vi/bible/1638/GEN.3.KTHD)</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-vai-goc-nhin-tu-thi-nghiem-vu-tru-25"&gt;Một vài góc nhìn từ thí nghiệm "Vũ trụ 25"&lt;/h1&gt;
 &lt;p&gt;Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi mãi hay không?  &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; Ông chọn ra 4 cặp chuột khỏe mạnh đã được sàng lọc kỹ càng về sức khỏe. Sau đó, đưa chúng vào môi trường 3m x 4.3m, chia thành 16 tháp, tạo được thành 256 hộp tổ, mỗi hộp có sức chứa đủ cho 15 chuột cùng ở - thiên đường đủ để chứa 4000 con chuột. Thức ăn, nước đều được cung cấp đầy đủ, nhiệt độ môi trường được kiểm soát, chất thải của chúng cũng được dọn dẹp, và hoàn toàn không có thú săn mồi. &lt;/p&gt;
@@ -2188,50 +2252,50 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Nói về bán hàng</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>noi-ve-ban-hang</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>26-07-2026</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51...</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>data\blogs\Nói về bán hàng.md</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t># Nói về bán hàng
 Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51 thứ tiếng và xuất hiện ở 109 quốc gia. Robert Kiyosaki có lần chia sẻ về câu chuyện hỏi người cha nuôi của mình tên Tommy cách để giàu như cha ông: 
@@ -2253,7 +2317,7 @@
 - [ ] Kỹ năng</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>&lt;h1 id="noi-ve-ban-hang"&gt;Nói về bán hàng&lt;/h1&gt;
 &lt;p&gt;Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51 thứ tiếng và xuất hiện ở 109 quốc gia. Robert Kiyosaki có lần chia sẻ về câu chuyện hỏi người cha nuôi của mình tên Tommy cách để giàu như cha ông: &lt;/p&gt;
@@ -2282,54 +2346,54 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Sách self-help có thật sự hữu ích?</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>sach-self-help-co-that-su-huu-ich</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
         <is>
           <t>10-06-2026</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>12-06-2026</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có...</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>data\blogs\Sách self-help có thật sự hữu ích.md</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t># Sách self-help có thật sự hữu ích?
 Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có đặc điểm chung là bán chạy bởi dễ đọc - dễ hiểu nếu so với những cuốn giáo trình khô khan. Tiêu biểu những cuốn điển hình mà anh em có lẽ đã quá quen thuộc là Đắc nhân tâm, Những kẻ xuất chúng, Nghĩ giàu làm giàu, 7 thói quen để thành đạt, Atomic Habit… 
@@ -2356,7 +2420,7 @@
 Một lần nữa, Hải muốn nhấn mạnh rằng: “Tri thức không chỉ phát triển nhờ sự đồng thuận tuyệt đối, mà nhờ những cuộc đối thoại tử tế. Vì vậy, mong anh em đọc bài viết như một góc nhìn để suy ngẫm, thay vì một kết luận cuối cùng. Mọi quan điểm ít nhiều đều mang dấu vết của trải nghiệm cá nhân. Mục đích của mỗi bài viết không phải là để ai đúng tuyệt đối, mà là liệu chúng ta có thể cùng nhau suy nghĩ sâu hơn sau mỗi bài viết hay không? Vì vậy, hãy đọc với tinh thần cởi mở và phản biện hoặc góp ý khi anh em có suy nghĩ khác nha!”.</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>&lt;h1 id="sach-self-help-co-that-su-huu-ich"&gt;Sách self-help có thật sự hữu ích?&lt;/h1&gt;
 &lt;p&gt;Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có đặc điểm chung là bán chạy bởi dễ đọc - dễ hiểu nếu so với những cuốn giáo trình khô khan. Tiêu biểu những cuốn điển hình mà anh em có lẽ đã quá quen thuộc là Đắc nhân tâm, Những kẻ xuất chúng, Nghĩ giàu làm giàu, 7 thói quen để thành đạt, Atomic Habit… &lt;/p&gt;
@@ -2384,57 +2448,15 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Thử thay đổi cách đặt câu hỏi</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>thu-thay-doi-cach-dat-cau-hoi</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>09-07-2026</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>10-07-2026</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>data\blogs\Thử thay đổi cách đặt câu hỏi.md</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-    </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Thử thay đổi góc nhìn</t>
+          <t>Thử thay đổi cách đặt câu hỏi</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>thu-thay-doi-goc-nhin</t>
+          <t>thu-thay-doi-cach-dat-cau-hoi</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2459,17 +2481,59 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>data\blogs\Thử thay đổi cách đặt câu hỏi.md</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Thử thay đổi góc nhìn</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>thu-thay-doi-goc-nhin</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>09-07-2026</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>10-07-2026</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành....</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>data\blogs\Thử thay đổi góc nhìn.md</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t># Thử thay đổi góc nhìn
 Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành. Anh ta luôn tự hào mình làm việc chăm chỉ. Cho tới một ngày, một sự cố ập đến, anh ta bị bệnh nặng và phải nhập viện. Sau gần 3 tháng điều trị, anh ta cũng đã khỏi bệnh. Vì không có bảo hiểm, tổng chi phí cho hóa đơn dài hơn 100 trang gồm tiền giường, tiền thuốc, tiền mổ và loạt chi phí khác đã chạm ngưỡng 1 triệu đô. Và tất nhiên, số tiền anh ta dành giụm rất nhỏ khi so với chi phí điều trị. Người từng tự đắc rằng mình không bao giờ nợ ai bất kỳ điều gì trên đời này cuối cùng lại nhận món nợ 1 triệu đô theo một cách mà không ai ngờ tới - viện phí.
@@ -2477,7 +2541,7 @@
 ## Thật ra tất cả mọi thứ còn tồn tại là vì còn nợ</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>&lt;h1 id="thu-thay-oi-goc-nhin"&gt;Thử thay đổi góc nhìn&lt;/h1&gt;
 &lt;p&gt;Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành. Anh ta luôn tự hào mình làm việc chăm chỉ. Cho tới một ngày, một sự cố ập đến, anh ta bị bệnh nặng và phải nhập viện. Sau gần 3 tháng điều trị, anh ta cũng đã khỏi bệnh. Vì không có bảo hiểm, tổng chi phí cho hóa đơn dài hơn 100 trang gồm tiền giường, tiền thuốc, tiền mổ và loạt chi phí khác đã chạm ngưỡng 1 triệu đô. Và tất nhiên, số tiền anh ta dành giụm rất nhỏ khi so với chi phí điều trị. Người từng tự đắc rằng mình không bao giờ nợ ai bất kỳ điều gì trên đời này cuối cùng lại nhận món nợ 1 triệu đô theo một cách mà không ai ngờ tới - viện phí.&lt;/p&gt;
@@ -2486,50 +2550,50 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Tài sản lớn nhất của một người</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>tai-san-lon-nhat-cua-mot-nguoi</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều th...</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>data\blogs\Tài sản lớn nhất của một người.md</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t># Tài sản lớn nhất của một người
 Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều thứ. Có người chấp nhận làm ăn xa xứ. Có người bỏ thời gian 8 - 16 tiếng mỗi ngày để làm việc. Có người nâng cao giá trị bản thân để kiếm nhiều tiền hơn. 
@@ -2585,7 +2649,7 @@
 Tuy nhiên, cũng nên lưu ý rằng câu **"Tài sản lớn nhất của một người là sự uy tín"** là một nhận định mang tính giá trị, không phải chân lý tuyệt đối. Với người khác, họ có thể cho rằng sức khỏe, thời gian hay tri thức mới là tài sản lớn nhất. Điều hợp lý hơn là xem **uy tín là một trong những tài sản vô hình giá trị nhất**, đặc biệt trong kinh doanh, lãnh đạo và các mối quan hệ lâu dài.</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-san-lon-nhat-cua-mot-nguoi"&gt;Tài sản lớn nhất của một người&lt;/h1&gt;
 &lt;p&gt;Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều thứ. Có người chấp nhận làm ăn xa xứ. Có người bỏ thời gian 8 - 16 tiếng mỗi ngày để làm việc. Có người nâng cao giá trị bản thân để kiếm nhiều tiền hơn. &lt;/p&gt;
@@ -2691,54 +2755,54 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Tâm lý học blogger - Tại sao Hải viết blog?</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>tam-ly-hoc-blogger---tai-sao-hai-viet-blog</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
         <is>
           <t>web, blog</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>01-06-2026</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và...</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học blogger -Tại sao Hải viết blog.md</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t># Tâm lý học blogger - Tại sao Hải lập blog riêng?
 Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và ghi lại để bất kỳ ai có thể xem lại sau này. Tất cả người xem bóng đá đều biết Mbappe, biết khả năng chơi bóng của anh ta, biết tốc độ của anh ta. Hàng loạt câu lạc bộ lớn muốn ký hợp đồng với anh ta với mức giá không tưởng.
@@ -2774,7 +2838,7 @@
 ---</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-blogger-tai-sao-hai-lap-blog-rieng"&gt;Tâm lý học blogger - Tại sao Hải lập blog riêng?&lt;/h1&gt;
 &lt;p&gt;Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và ghi lại để bất kỳ ai có thể xem lại sau này. Tất cả người xem bóng đá đều biết Mbappe, biết khả năng chơi bóng của anh ta, biết tốc độ của anh ta. Hàng loạt câu lạc bộ lớn muốn ký hợp đồng với anh ta với mức giá không tưởng.&lt;/p&gt;
@@ -2811,84 +2875,84 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Tâm lý học cá độ - Vì sao người không chơi là người thắng</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-ca-do---vi-sao-nguoi-khong-choi-la-nguoi-thang</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>08-06-2026</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>02-07-2026</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học cá độ - Vì sao người không chơi là người thắng.md</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-    </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tâm lý học của người lười nhưng tham vọng lớn</t>
+          <t>Tâm lý học cá độ - Vì sao người không chơi là người thắng</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-cua-nguoi-luoi-nhung-tham-vong-lon</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Tâm lý</t>
-        </is>
-      </c>
+          <t>tam-ly-hoc-ca-do---vi-sao-nguoi-khong-choi-la-nguoi-thang</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
+          <t>08-06-2026</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học cá độ - Vì sao người không chơi là người thắng.md</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tâm lý học của người lười nhưng tham vọng lớn</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>tam-ly-hoc-cua-nguoi-luoi-nhung-tham-vong-lon</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Tâm lý</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
           <t>26-05-2026</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xu...</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học của người lười nhưng tham vọng đạt được thành tựu lớn.md</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t># Tâm lý học của người lười nhưng tham vọng lớn
 Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xuất hiện trong hàng triệu triệu người mỗi ngày. Đó chính là tâm lý của người lười nhưng tham vọng lớn. 
@@ -2917,7 +2981,7 @@
 Giáo sư Jiang Xue Qin</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-cua-nguoi-luoi-nhung-tham-vong-lon"&gt;Tâm lý học của người lười nhưng tham vọng lớn&lt;/h1&gt;
 &lt;p&gt;Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xuất hiện trong hàng triệu triệu người mỗi ngày. Đó chính là tâm lý của người lười nhưng tham vọng lớn. &lt;/p&gt;
@@ -2947,54 +3011,54 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Tâm lý học FOMO</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>tam-ly-hoc-fomo</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
         <is>
           <t>fomo</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>28-05-2026</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành...</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học FOMO.md</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t># Tâm lý học FOMO
 Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành viên đó sẽ gặp nguy hiểm. Ngày nay, chúng ta thấy tâm lý FOMO (fear-of-missing-out) ở khắp mọi nơi: cái áo chỉ giảm giá trong ngày, drama trên mạng xã hội, sóng đầu tư tiền ảo, tin tức thời sự,... Khai thác FOMO là ngành công nghiệp kiếm rất nhiều tiền bởi con người không chỉ sợ thất bại, họ còn sợ mình đang đứng yên trong khi người khác vẫn chạy.
@@ -3017,7 +3081,7 @@
 FOMO không phải dấu hiệu của sự nhu nhược, hay sự thiếu quyết đoán. Nó là phản ứng rất bình thường của não bộ con người từ xưa tới nay. Từ thời kỳ săn bắt hái lượm tới thời kỳ drama và trào lưu trên mạng xã hội. Xóa bỏ hoàn toàn tâm lý FOMO là vô ích và tự hủy cơ chế bảo vệ bản thân mà tạo hóa ban tặng.</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-fomo"&gt;Tâm lý học FOMO&lt;/h1&gt;
 &lt;p&gt;Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành viên đó sẽ gặp nguy hiểm. Ngày nay, chúng ta thấy tâm lý FOMO (fear-of-missing-out) ở khắp mọi nơi: cái áo chỉ giảm giá trong ngày, drama trên mạng xã hội, sóng đầu tư tiền ảo, tin tức thời sự,... Khai thác FOMO là ngành công nghiệp kiếm rất nhiều tiền bởi con người không chỉ sợ thất bại, họ còn sợ mình đang đứng yên trong khi người khác vẫn chạy.&lt;/p&gt;
@@ -3041,49 +3105,49 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Tâm lý học kinh nghiệm</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>tam-ly-hoc-kinh-nghiem</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>Anh đọc bài viết em cũng ổn.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học kinh nghiệm.md</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Anh đọc bài viết em cũng ổn.
 Ví dụ tâm lý học nhà thầu, em phân tích mục đích và hành động của nhiều nhóm người chơi nhưng không đưa ra được hệ phương trình vi phân để mô hình hóa sự thay đổi động lực của các người chơi trong dự án. Em cũng không đưa ra được mô hình xác suất có điều kiện trong trường hợp nào nhà thầu sẽ ưu tiên tìm đối tác giá rẻ và trong trường hợp nào họ ưu tiên sự yên tâm. 
 Hay 1 ví dụ khác</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>&lt;p&gt;Anh đọc bài viết em cũng ổn.&lt;/p&gt;
 &lt;p&gt;Ví dụ tâm lý học nhà thầu, em phân tích mục đích và hành động của nhiều nhóm người chơi nhưng không đưa ra được hệ phương trình vi phân để mô hình hóa sự thay đổi động lực của các người chơi trong dự án. Em cũng không đưa ra được mô hình xác suất có điều kiện trong trường hợp nào nhà thầu sẽ ưu tiên tìm đối tác giá rẻ và trong trường hợp nào họ ưu tiên sự yên tâm. &lt;/p&gt;
@@ -3091,50 +3155,50 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Tâm lý học Michelin Boy</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>tam-ly-hoc-michelin-boy</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>indraft</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>07-06-2026</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học Michelin Boy.md</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t># Tâm lý học Michelin Boy
 Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.
@@ -3157,7 +3221,7 @@
 [^1]: This is the footnote.</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-michelin-boy"&gt;Tâm lý học Michelin Boy&lt;/h1&gt;
 &lt;p&gt;Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.&lt;/p&gt;
@@ -3186,69 +3250,15 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Tâm lý học một view</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-mot-view</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Tâm lý</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>20-07-2026</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>20-07-2026</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học một view.md</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t># Tâm lý học một view</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>&lt;h1 id="tam-ly-hoc-mot-view"&gt;Tâm lý học một view&lt;/h1&gt;</t>
-        </is>
-      </c>
-    </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Tâm lý học nghiện xem video phát triển bản thân</t>
+          <t>Tâm lý học một view</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-nghien-xem-video-phat-trien-ban-than</t>
+          <t>tam-ly-hoc-mot-view</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3256,30 +3266,84 @@
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Tâm lý</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học một view.md</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t># Tâm lý học một view</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="tam-ly-hoc-mot-view"&gt;Tâm lý học một view&lt;/h1&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tâm lý học nghiện xem video phát triển bản thân</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tam-ly-hoc-nghien-xem-video-phat-trien-ban-than</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>29-05-2026</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>30-05-2026</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nh...</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học nghiện xem video phát triển bản thân.md</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t># Tâm lý học nghiện xem video phát triển bản thân
 Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nhằm 1 mục đích là nâng cấp bản thân. Cũng từ đó, có một thứ nghiện khá mới trong thời đại mạng xã hội ngày nay, không phải nghiện game, không phải nghiện phim mà là nghiện xem video phát triển bản thân. 
@@ -3290,7 +3354,7 @@
 ##</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nghien-xem-video-phat-trien-ban-than"&gt;Tâm lý học nghiện xem video phát triển bản thân&lt;/h1&gt;
 &lt;p&gt;Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nhằm 1 mục đích là nâng cấp bản thân. Cũng từ đó, có một thứ nghiện khá mới trong thời đại mạng xã hội ngày nay, không phải nghiện game, không phải nghiện phim mà là nghiện xem video phát triển bản thân. &lt;/p&gt;
@@ -3302,58 +3366,58 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Tâm lý học ngành bột mì</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nganh-bot-mi</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>bột mì</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>28-05-2026</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã c...</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học ngành bột mì.md</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t># Tâm lý học ngành bột mì
 Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã có gần như tất cả mọi thứ lại dính vào thứ tệ nạn này? Và tại sao trong rất nhiều thập kỷ, ngành công nghiệp này vẫn tồn tại bất kể luật pháp trừng phạt rất mạnh tay?
@@ -3390,7 +3454,7 @@
 Đứng trước lợi nhuận khổng lồ, nhiều cá nhân chấp nhận rủi ro đối mặt án tử để đi sản xuất, tàng trữ và vận chuyển bột mì. Và tất nhiên, phía bên kia của lợi nhuận đó chính là những cuộc đời bị phá hủy, những gia đình tan vỡ, những người trẻ đánh mất tương lai. Bản thân ngành công nghiệp bột mì còn tồn tại không phải chỉ nằm ở việc nó là chất kích thích, nó khai thác vào cảm giác cô đơn, áp lực, muốn hòa nhập, muốn thoát khỏi thực tại của mỗi người. Nó không chỉ là câu chuyện của pháp luật, nó còn là câu chuyện của giáo dục, môi trường sống và các mối quan hệ.</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nganh-bot-mi"&gt;Tâm lý học ngành bột mì&lt;/h1&gt;
 &lt;p&gt;Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã có gần như tất cả mọi thứ lại dính vào thứ tệ nạn này? Và tại sao trong rất nhiều thập kỷ, ngành công nghiệp này vẫn tồn tại bất kể luật pháp trừng phạt rất mạnh tay?&lt;/p&gt;
@@ -3453,58 +3517,58 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Tâm lý học nhà thầu</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nha-thau</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>thầu, dự án</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>26-05-2026</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu...</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học nhà thầu.md</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t># Tâm lý học nhà thầu
 Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu. Một kỹ sư hiện trường sẽ có góc nhìn khác đơn vị thiết kế. Một công nhân sẽ có góc nhìn khác người quản lý dự án. Vì vậy, bài viết chỉ là một góc nhìn của Hải dưới lăng kính tâm lý học và lý thuyết trò chơi.
@@ -3549,7 +3613,7 @@
 Bài viết này chủ yếu được nhìn dưới lăng kính tâm lý học, kinh tế học và lý thuyết trò chơi. Hải hiểu rằng thực tế ngoài công trường luôn phức tạp hơn rất nhiều so với những gì có thể trình bày trong một bài blog. Nên nếu anh em đang làm trong lĩnh vực xây dựng, đấu thầu, quản lý dự án, giám sát, thiết kế hoặc từng tham gia các dự án lớn, Hải rất mong nhận được những góp ý, phản biện hoặc góc nhìn khác của anh em qua email **nguyenquyhai2002@gmail.com**.</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nha-thau"&gt;Tâm lý học nhà thầu&lt;/h1&gt;
 &lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu. Một kỹ sư hiện trường sẽ có góc nhìn khác đơn vị thiết kế. Một công nhân sẽ có góc nhìn khác người quản lý dự án. Vì vậy, bài viết chỉ là một góc nhìn của Hải dưới lăng kính tâm lý học và lý thuyết trò chơi.&lt;/p&gt;
@@ -3632,49 +3696,15 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Tâm lý học phông bạt</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-phong-bat</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học phông bạt.md</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-    </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Tâm lý học sưu tầm tài liệu nhưng không đọc</t>
+          <t>Tâm lý học phông bạt</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-suu-tam-tai-lieu-nhung-khong-doc</t>
+          <t>tam-ly-hoc-phong-bat</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -3683,18 +3713,18 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>29-05-2026</t>
+          <t>26-05-2026</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>29-05-2026</t>
+          <t>26-05-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>data\blogs\Tâm lý học sưu tầm tài liệu nhưng không đọc.md</t>
+          <t>data\blogs\Tâm lý học phông bạt.md</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -3703,12 +3733,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người</t>
+          <t>Tâm lý học sưu tầm tài liệu nhưng không đọc</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-trai-tim-em-nho-lam-nen-chi-chua-duoc-mot-nguoi</t>
+          <t>tam-ly-hoc-suu-tam-tai-lieu-nhung-khong-doc</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -3717,50 +3747,32 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>26-05-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học l...</t>
-        </is>
-      </c>
+          <t>29-05-2026</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>data\blogs\Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người.md</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.
-## Cảm xúc mới lạ
-## Tại sao chúng ta không bao giờ đọc
-##</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.&lt;/p&gt;
-&lt;h2 id="cam-xuc-moi-la"&gt;Cảm xúc mới lạ&lt;/h2&gt;
-&lt;h2 id="tai-sao-chung-ta-khong-bao-gio-oc"&gt;Tại sao chúng ta không bao giờ đọc&lt;/h2&gt;
-&lt;h2 id="_1"&gt;&lt;/h2&gt;</t>
-        </is>
-      </c>
+          <t>data\blogs\Tâm lý học sưu tầm tài liệu nhưng không đọc.md</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm</t>
+          <t>Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-xo-so---vi-sao-nguoi-trung-so-thuong-ve-no-sau-vai-nam</t>
+          <t>tam-ly-hoc-trai-tim-em-nho-lam-nen-chi-chua-duoc-mot-nguoi</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -3774,66 +3786,118 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
+          <t>08-06-2026</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học l...</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>data\blogs\Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm.md</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+          <t>data\blogs\Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người.md</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.
+## Cảm xúc mới lạ
+## Tại sao chúng ta không bao giờ đọc
+##</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.&lt;/p&gt;
+&lt;h2 id="cam-xuc-moi-la"&gt;Cảm xúc mới lạ&lt;/h2&gt;
+&lt;h2 id="tai-sao-chung-ta-khong-bao-gio-oc"&gt;Tại sao chúng ta không bao giờ đọc&lt;/h2&gt;
+&lt;h2 id="_1"&gt;&lt;/h2&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tìm hiểu về MCP</t>
+          <t>Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>tim-hieu-ve-mcp</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Công nghệ</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
+          <t>tam-ly-hoc-xo-so---vi-sao-nguoi-trung-so-thuong-ve-no-sau-vai-nam</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm.md</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Tìm hiểu về MCP</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>tim-hieu-ve-mcp</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
           <t>06-07-2026</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>15-07-2026</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>Hãy bắt đầu với 1 công cụ mà chúng ta đều biết - ChatGPT. Khi 1 người muốn nhờ ChatGPT làm 1 điều gì đó, họ sẽ gửi prompt và sau đó ChatGPT sẽ phản hồi lại người đó. Và xuyên suốt quá trình này chỉ nhận văn bản và trả về văn bản. Không có 1...</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>data\blogs\Tìm hiểu về MCP.md</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t># Tìm hiểu về MCP
 ## Tại sao chúng ta cần MCP
@@ -3844,7 +3908,7 @@
 *MCP như cổng kết nối USB. Nguồn: modelcontextprotocol.io*</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>&lt;h1 id="tim-hieu-ve-mcp"&gt;Tìm hiểu về MCP&lt;/h1&gt;
 &lt;h2 id="tai-sao-chung-ta-can-mcp"&gt;Tại sao chúng ta cần MCP&lt;/h2&gt;
@@ -3856,50 +3920,50 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Tư duy cắt chuỗi</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>tu-duy-cat-chuoi</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ...</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy cắt chuỗi.md</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t># Tư duy cắt chuỗi
 Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ trợ chúng ta có nền tảng để tự dụng lên mọi nội dung, hệ thống. Nó chính là bước khác biệt và cũng là bước khó nhất trong toàn bộ quy trình tự động.   
@@ -3914,7 +3978,7 @@
 ## Kết</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-cat-chuoi"&gt;Tư duy cắt chuỗi&lt;/h1&gt;
 &lt;p&gt;Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ trợ chúng ta có nền tảng để tự dụng lên mọi nội dung, hệ thống. Nó chính là bước khác biệt và cũng là bước khó nhất trong toàn bộ quy trình tự động.   &lt;/p&gt;
@@ -3930,62 +3994,20 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Tư duy Excel</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>tu-duy-excel</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>08-06-2026</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>08-06-2026</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>data\blogs\Tư duy Excel.md</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-    </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tư duy ngược và tư duy mở ngành phần mềm</t>
+          <t>Tư duy Excel</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>tu-duy-nguoc-va-tu-duy-mo-nganh-phan-mem</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
+          <t>tu-duy-excel</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
@@ -3997,17 +4019,59 @@
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>data\blogs\Tư duy Excel.md</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Tư duy ngược và tư duy mở ngành phần mềm</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>tu-duy-nguoc-va-tu-duy-mo-nganh-phan-mem</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>08-06-2026</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>08-06-2026</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
         <is>
           <t>Linux - Windows - Mac</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy ngược và tư duy mở ngành phần mềm.md</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t># Tư duy ngược và tư duy mở ngành phần mềm
 ## Những thứ có giá trị nhất đôi khi là rẻ nhất hoặc miễn phí
@@ -4016,7 +4080,7 @@
 ## Giải pháp triệu đô</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-nguoc-va-tu-duy-mo-nganh-phan-mem"&gt;Tư duy ngược và tư duy mở ngành phần mềm&lt;/h1&gt;
 &lt;h2 id="nhung-thu-co-gia-tri-nhat-oi-khi-la-re-nhat-hoac-mien-phi"&gt;Những thứ có giá trị nhất đôi khi là rẻ nhất hoặc miễn phí&lt;/h2&gt;
@@ -4026,58 +4090,58 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Tư duy xô nước</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>tu-duy-xo-nuoc</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Tư duy</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>xô nước, đường ống</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>16-06-2026</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến....</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy xô nước.md</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t># Tư duy xô nước
 Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến.  Giai đoạn đầu, các thanh niên trong làng hứng khởi và xách xô nước vì số tiền họ kiếm được phụ thuộc vào số xô nước họ giao. Các gia đình ai ai cũng muốn gả con gái cho những thanh niên chăm chỉ sẵn sàng đi xách nước vào cả khung giờ chiều tối, nửa đêm để đáp ứng nhu cầu sử dụng nước cho nhiều gia đình. Sự thành đạt, tinh thần làm việc chăm chỉ, tương lai cầu tiến được thể hiện bằng số giờ đi xách xô nước và số xô nước họ đã mang đến từng nhà. Các thanh niên ốm yếu, gầy gò trong làng lúc này cũng đã tham gia vì công việc này ngày nào cũng có và không hết việc. Và đó cũng là việc mà các thanh thiếu niên chí khí trong làng lúc bấy giờ nên dấn thân. 
@@ -4107,7 +4171,7 @@
 Một trong những thứ có thể tồn tại lâu hơn tuổi thọ của con người đó là đường ống. Con người rồi sẽ già đi. Sức khỏe rồi sẽ suy giảm. Thời gian của mỗi người đều có giới hạn. Nhưng những gì chúng ta để lại thì không nhất thiết phải biến mất. Ai cũng có thể phải xách xô ở một giai đoạn nào đó của cuộc đời. Không có gì đáng xấu hổ khi dùng thời gian và sức lao động để kiếm sống. Vấn đề chỉ nằm ở chỗ: liệu sau mỗi ngày xách xô, chúng ta có dành ra một phần thời gian để xây đường ống hay không? Bởi vì đến một lúc nào đó, thứ quyết định giá trị của một con người không còn là họ đã đổ bao nhiêu mồ hôi, thức bao nhiêu đêm hay làm việc bao nhiêu giờ mỗi ngày, mà là những gì vẫn tiếp tục tạo ra giá trị ngay cả khi họ không còn ở đó.</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-xo-nuoc"&gt;Tư duy xô nước&lt;/h1&gt;
 &lt;p&gt;Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến.  Giai đoạn đầu, các thanh niên trong làng hứng khởi và xách xô nước vì số tiền họ kiếm được phụ thuộc vào số xô nước họ giao. Các gia đình ai ai cũng muốn gả con gái cho những thanh niên chăm chỉ sẵn sàng đi xách nước vào cả khung giờ chiều tối, nửa đêm để đáp ứng nhu cầu sử dụng nước cho nhiều gia đình. Sự thành đạt, tinh thần làm việc chăm chỉ, tương lai cầu tiến được thể hiện bằng số giờ đi xách xô nước và số xô nước họ đã mang đến từng nhà. Các thanh niên ốm yếu, gầy gò trong làng lúc này cũng đã tham gia vì công việc này ngày nào cũng có và không hết việc. Và đó cũng là việc mà các thanh thiếu niên chí khí trong làng lúc bấy giờ nên dấn thân. &lt;/p&gt;
@@ -4138,54 +4202,54 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Tại sao Bitcoin cưa đôi?</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>tai-sao-bitcoin-cua-doi</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải...</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>data\blogs\Tại sao Bitcon cưa đôi.md</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t># Tại sao Bitcoin cưa đôi?
 Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?
@@ -4251,7 +4315,7 @@
 [^3]: [Controlled supply - Bitcoin Wiki](https://en.bitcoin.it/wiki/Controlled_supply)</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-bitcoin-cua-oi"&gt;Tại sao Bitcoin cưa đôi?&lt;/h1&gt;
 &lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?&lt;/p&gt;
@@ -4307,11 +4371,13 @@
 &lt;p&gt;Phần thưởng khi đào được quy đổi ra Bitcoin sẽ có xu hướng giảm như công thức trên. Cứ sau mỗi giai đoạn, phần thưởng khi đào được sẽ bị cưa đôi. Cứ sau mỗi chu kỳ, phần thưởng coin dành cho người đào được sẽ giảm đi một nửa. Cha đẻ của Bitcoin làm vậy để đảm bảo rằng tổng số Bitcoin sẽ giới hạn ở con số 21 triệu. &lt;sup id="fnref:3"&gt;&lt;a class="footnote-ref" href="#fn:3"&gt;3&lt;/a&gt;&lt;/sup&gt;&lt;/p&gt;
 &lt;p&gt;Vậy cha đẻ của Bitcoin là Satoshi Nakamoto có biết trước về chỗ chứa các Bitcoin chưa được khai phá hay không? Câu trả lời là ông hoàn toàn không biết, trừ khi ông chọn cách đào như những người khác. Dù ông biết thuật toán, biết cơ chế tạo block, biết kiểm tra PoW, nhưng ông không khác gì những người bình thường khác vì những gì ông biết đều được công khai trên mã nguồn mở. Cái số mà các thợ đào coin phải tìm nó chưa từng được ai đó đẻ ra. Số đó chỉ có thể đi tìm và dùng để thử sai tới khi khớp chuỗi. Hệ thống không hề tạo ra số nonce ngẫu nhiên mà mà tạo ra kết quả băm ngẫu nhiên dể mọi người tìm số nounce phù hợp. Ngay cả khi anh em giỏi đến mức biết được seed random, anh em cũng không thể kiểm soát được nội dung và thời điểm giao dịch trong tương lai, và vì thế, không thể biết được chuỗi tiếp theo và càng không thể biết được số nounce nếu như không thử sai. &lt;/p&gt;
 &lt;h2 id="tuong-lai-cong-nghe-hay-chieu-tro-thoi-bong-bong"&gt;Tương lai công nghệ hay chiêu trò thổi bong bóng?&lt;/h2&gt;
-&lt;p&gt;Khi chúng ta đã đi qua 4 câu hỏi:
-- [x] Tư duy nào hình thành nên sổ cái phi tập trung?
-- [x] Làm sao để chuyển tiền?
-- [x] Làm sao để biết giao dịch có hợp lệ hay không?
-- [x] Tiền hay số dư của Bitcoin đến từ đâu?&lt;/p&gt;
+&lt;p&gt;Khi chúng ta đã đi qua 4 câu hỏi:&lt;/p&gt;
+&lt;ul class="task-list"&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox" checked/&gt; Tư duy nào hình thành nên sổ cái phi tập trung?&lt;/li&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox" checked/&gt; Làm sao để chuyển tiền?&lt;/li&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox" checked/&gt; Làm sao để biết giao dịch có hợp lệ hay không?&lt;/li&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox" checked/&gt; Tiền hay số dư của Bitcoin đến từ đâu?&lt;/li&gt;
+&lt;/ul&gt;
 &lt;p&gt;Chúng ta vẫn sẽ còn rất nhiều câu hỏi về giá trị của Bitcoin. Chúng không thể làm trang sức như vàng, cũng không thể làm chỗ ở hay mặt bằng kinh doanh như đất, cũng không phải là dạng đầu tư cho sản xuất như cổ phiếu, cũng không được chính phủ coi như tiền mặt chính thống. Vậy một thứ không thể cầm nắm, không thể sờ, không thể ngửi như Bitcoin thì có giá trị gì? Tại sao 1 Bitcoin quy đổi ra USD lại có giá trị khủng khiếp như vậy? Nó sẽ tăng hay giảm trong tương lai? Điều này liệu sẽ sụp đổ? &lt;/p&gt;
 &lt;p&gt;Như Hải đã trình bày, bản chất của Bitcoin là ghi nhận giao dịch. Tất cả giao dịch được công nhận đều được lưu trên nhiều hệ thống khác nhau và đồng bộ với nhau nên giá trị của nó là đảm bảo các bên nhớ được giao dịch. Về lượng cung, Bitcoin có giới hạn giống như đất đai và vàng, không ai có thể tạo ra thêm Bitcoin. Và đó là lý do tỷ giá Bitcoin so với đồng tiền của hầu hết quốc gia luôn biến động rất mạnh vì lạm phát của tiền truyền thống và vì nhu cầu sở hữu Bitcoin luôn thay đổi. Và cũng có cả sự đầu cơ và thao túng truyền thông làm giá Bitcoin nhảy lên xuống liên tục nữa. Nhưng về dài hạn, lượng tiền mỗi quốc gia có khuynh hướng phát hành thêm, nhân khẩu có xu hướng tăng, năng suất lao động tăng, hiệu quả sản xuất luôn đi lên do tiến bộ về khoa học và công nghệ. Và dù những thứ trên có tăng bao nhiêu đi chăng nữa thì số lượng Bitcoin vẫn không tăng, nên Bitoin vẫn có khả năng tăng giá như đất đai hay vàng. Và chính vì chúng không nằm cố định một chỗ như đất đai, không phải ký gửi hành lý hay kiểm tra khi đi qua an ninh sân bay như vàng, chúng có giá trị riêng là có thể chảy đến bất kỳ đâu, chuyển tới bất kỳ đâu, không phân biệt người gửi/nhận là ai và cũng không chịu sự ảnh hưởng của bất kỳ tổ chức nào. &lt;/p&gt;
 &lt;p&gt;Vì ai có Bitcoin cũng có thể chuyển Bitcoin cho bất kỳ ai, nên Bitcoin bị nhiều người lo ngại rằng sẽ được dùng cho các giao dịch phạm pháp hoặc là rửa tiền. Nhưng quay lại với bản chất của Bitcoin một lần nữa, nó được sinh ra là để giải quyết bài toán ghi chép lại ai đã giao dịch với ai. Vì thế, mọi giao dịch đều được lưu lại và thống nhất ở nhiều nơi. Dù có thể không biết ai đứng đằng sau ví, mọi người đều có thể biết được giao dịch và phân tích khoanh vùng nếu họ thật sự muốn. Và vì thế, nếu muốn biết Bitcoin là tương lai nhân loại hay trò thổi bong bóng, hãy hỏi điều tương tự với mỗi hệ thống tài chính và tiền tệ từ mỗi quốc gia anh em đã và đang sinh sống câu hỏi tương tự mà anh em đã đặt cho Bitcoin:
@@ -4339,69 +4405,15 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Tại sao lại là Blockchain</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>tai-sao-lai-la-blockchain</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Công nghệ</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>20-07-2026</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>20-07-2026</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>data\blogs\Tại sao lại là Blockchain.md</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t># Tại sao lại là Blockchain?</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>&lt;h1 id="tai-sao-lai-la-blockchain"&gt;Tại sao lại là Blockchain?&lt;/h1&gt;</t>
-        </is>
-      </c>
-    </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vì sao con người tự ti</t>
+          <t>Tại sao lại là Blockchain</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>vi-sao-con-nguoi-tu-ti</t>
+          <t>tai-sao-lai-la-blockchain</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4409,7 +4421,11 @@
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
@@ -4418,31 +4434,81 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>data\blogs\Tại sao lại là Blockchain.md</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t># Tại sao lại là Blockchain?</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="tai-sao-lai-la-blockchain"&gt;Tại sao lại là Blockchain?&lt;/h1&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Vì sao con người tự ti</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>vi-sao-con-nguoi-tu-ti</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>- [ ] họ không tự hào về bản thân họ, về môi trường họ sinh ra, về</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao con người tự ti.md</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t># Vì sao con người tự ti?
 - [ ] họ không tự hào về bản thân họ, về môi trường họ sinh ra, về</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>&lt;h1 id="vi-sao-con-nguoi-tu-ti"&gt;Vì sao con người tự ti?&lt;/h1&gt;
 &lt;ul class="task-list"&gt;
@@ -4451,84 +4517,84 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Vì sao khởi nghiệp thất bại</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>vi-sao-khoi-nghiep-that-bai</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>20-07-2026</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>20-07-2026</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>data\blogs\Vì sao khởi nghiệp thất bại.md</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-    </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Vì sao người giàu thích nợ?</t>
+          <t>Vì sao khởi nghiệp thất bại</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>vi-sao-nguoi-giau-thich-no</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+          <t>vi-sao-khoi-nghiep-that-bai</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>data\blogs\Vì sao khởi nghiệp thất bại.md</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Vì sao người giàu thích nợ?</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>vi-sao-nguoi-giau-thich-no</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>02-07-2026</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết n...</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao người giàu thích nợ.md</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t># Vì sao người giàu thích nợ
 Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết người đàn ông đó là ai không?”. “Em biết, ông ấy là ăn xin” - cô gái đáp. Ông Trump nói tiếp: “Ngay bây giờ, ông ấy đang có nhiều hơn anh 900 triệu đô”. Và cô gái thắc mắc: “Làm sao người ăn xin có thể có nhiều tiền hơn ông được?”. Bởi vì người ăn xin tuy  không có đồng nào nhưng cũng không có nợ. Trong khi đó, ông Trump nợ 900 triệu đô. Đó là thời điểm bất động sản ở Mỹ đang ở dưới đáy chu kỳ vào những năm đầu thập niên 90. Và tất nhiên sau đó, thị trường bất động sản ở New York mà ông Trump đầu tư xây dựng đã phát triển bùng nổ.
@@ -4563,7 +4629,7 @@
 Cái gì quan trọng thì nhắc lại ba lần: “Ai sinh ra trên đời cũng chỉ có 2 bàn tay trắng và sẽ không cầm theo được bất cứ thứ gì khi rời đi”. Nhìn nhận về nợ ra sao, đó là quan điểm của mỗi người. Chúng ta chỉ biết rằng, trong lịch sử loài người, nếu không có thứ đó, sẽ mất rất lâu nữa để có hàng ngàn sa số những công trình, công nghệ được xây dựng và phát triển tới tận ngày nay. Không có thứ đó, hàng triệu triệu người sẽ phải chôn vùi giấc mơ, những điều mình muốn làm và mang theo nó sang thế giới bên kia thay vì để lại cho nhân loại.</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>&lt;h1 id="vi-sao-nguoi-giau-thich-no"&gt;Vì sao người giàu thích nợ&lt;/h1&gt;
 &lt;p&gt;Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết người đàn ông đó là ai không?”. “Em biết, ông ấy là ăn xin” - cô gái đáp. Ông Trump nói tiếp: “Ngay bây giờ, ông ấy đang có nhiều hơn anh 900 triệu đô”. Và cô gái thắc mắc: “Làm sao người ăn xin có thể có nhiều tiền hơn ông được?”. Bởi vì người ăn xin tuy  không có đồng nào nhưng cũng không có nợ. Trong khi đó, ông Trump nợ 900 triệu đô. Đó là thời điểm bất động sản ở Mỹ đang ở dưới đáy chu kỳ vào những năm đầu thập niên 90. Và tất nhiên sau đó, thị trường bất động sản ở New York mà ông Trump đầu tư xây dựng đã phát triển bùng nổ.&lt;/p&gt;
@@ -4599,50 +4665,50 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Điều mà nhà trường không bao giờ nói với anh em</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>dieu-ma-nha-truong-khong-bao-gio-noi-voi-anh-em</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Kinh tế</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
         <is>
           <t>25-05-2026</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>Hầu hết chúng ta được dạy rằng, phải học thật giỏi, thi vào những trường tốt nhất thì mới có cơ hội vào được 1 công ty tốt. Sau đó làm việc thật chăm chỉ, 8 tiếng mỗi ngày, 5 ngày mỗi tuần, có thể chủ động xin tăng ca để tích lũy thêm tiền...</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>data\blogs\Điều mà nhà trường không bao giờ nói với anh em.md</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t># Điều mà nhà trường không bao giờ nói với anh em
 ## 2 kiểu tư duy về tiền
@@ -4689,7 +4755,7 @@
 Tâm lý học về tiền</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>&lt;h1 id="ieu-ma-nha-truong-khong-bao-gio-noi-voi-anh-em"&gt;Điều mà nhà trường không bao giờ nói với anh em&lt;/h1&gt;
 &lt;h2 id="2-kieu-tu-duy-ve-tien"&gt;2 kiểu tư duy về tiền&lt;/h2&gt;

</xml_diff>

<commit_message>
Edit Bitcoin blog post 2
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -427,7 +427,7 @@
     <col width="245" customWidth="1" min="9" max="9"/>
     <col width="103" customWidth="1" min="10" max="10"/>
     <col width="13838" customWidth="1" min="11" max="11"/>
-    <col width="16121" customWidth="1" min="12" max="12"/>
+    <col width="16181" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4380,14 +4380,16 @@
 &lt;/ul&gt;
 &lt;p&gt;Chúng ta vẫn sẽ còn rất nhiều câu hỏi về giá trị của Bitcoin. Chúng không thể làm trang sức như vàng, cũng không thể làm chỗ ở hay mặt bằng kinh doanh như đất, cũng không phải là dạng đầu tư cho sản xuất như cổ phiếu, cũng không được chính phủ coi như tiền mặt chính thống. Vậy một thứ không thể cầm nắm, không thể sờ, không thể ngửi như Bitcoin thì có giá trị gì? Tại sao 1 Bitcoin quy đổi ra USD lại có giá trị khủng khiếp như vậy? Nó sẽ tăng hay giảm trong tương lai? Điều này liệu sẽ sụp đổ? &lt;/p&gt;
 &lt;p&gt;Như Hải đã trình bày, bản chất của Bitcoin là ghi nhận giao dịch. Tất cả giao dịch được công nhận đều được lưu trên nhiều hệ thống khác nhau và đồng bộ với nhau nên giá trị của nó là đảm bảo các bên nhớ được giao dịch. Về lượng cung, Bitcoin có giới hạn giống như đất đai và vàng, không ai có thể tạo ra thêm Bitcoin. Và đó là lý do tỷ giá Bitcoin so với đồng tiền của hầu hết quốc gia luôn biến động rất mạnh vì lạm phát của tiền truyền thống và vì nhu cầu sở hữu Bitcoin luôn thay đổi. Và cũng có cả sự đầu cơ và thao túng truyền thông làm giá Bitcoin nhảy lên xuống liên tục nữa. Nhưng về dài hạn, lượng tiền mỗi quốc gia có khuynh hướng phát hành thêm, nhân khẩu có xu hướng tăng, năng suất lao động tăng, hiệu quả sản xuất luôn đi lên do tiến bộ về khoa học và công nghệ. Và dù những thứ trên có tăng bao nhiêu đi chăng nữa thì số lượng Bitcoin vẫn không tăng, nên Bitoin vẫn có khả năng tăng giá như đất đai hay vàng. Và chính vì chúng không nằm cố định một chỗ như đất đai, không phải ký gửi hành lý hay kiểm tra khi đi qua an ninh sân bay như vàng, chúng có giá trị riêng là có thể chảy đến bất kỳ đâu, chuyển tới bất kỳ đâu, không phân biệt người gửi/nhận là ai và cũng không chịu sự ảnh hưởng của bất kỳ tổ chức nào. &lt;/p&gt;
-&lt;p&gt;Vì ai có Bitcoin cũng có thể chuyển Bitcoin cho bất kỳ ai, nên Bitcoin bị nhiều người lo ngại rằng sẽ được dùng cho các giao dịch phạm pháp hoặc là rửa tiền. Nhưng quay lại với bản chất của Bitcoin một lần nữa, nó được sinh ra là để giải quyết bài toán ghi chép lại ai đã giao dịch với ai. Vì thế, mọi giao dịch đều được lưu lại và thống nhất ở nhiều nơi. Dù có thể không biết ai đứng đằng sau ví, mọi người đều có thể biết được giao dịch và phân tích khoanh vùng nếu họ thật sự muốn. Và vì thế, nếu muốn biết Bitcoin là tương lai nhân loại hay trò thổi bong bóng, hãy hỏi điều tương tự với mỗi hệ thống tài chính và tiền tệ từ mỗi quốc gia anh em đã và đang sinh sống câu hỏi tương tự mà anh em đã đặt cho Bitcoin:
-- Tiền đến từ đâu, tiền được tạo ra như thế nào?
-- Ai là người có quyền quyết định cung tiền? Ai là người kiểm soát cung tiền?
-- Giao dịch được ghi lại như thế nào?
-- Dòng tiền có minh bạch hay không, có sạch hay không?
-- Ở đâu bạn có 10 tỷ gửi tiết kiệm? 
-- Từ đâu bạn có tiền mua biệt thự, mua Maybach, mua Porsche? 
-- Nếu bạn làm mất địa chỉ ví cá nhân, bạn mất toàn bộ tài sản Bitcoin, vậy nếu như bạn đánh rơi ví tiền ở ngoài đường thì sao?&lt;/p&gt;
+&lt;p&gt;Vì ai có Bitcoin cũng có thể chuyển Bitcoin cho bất kỳ ai, nên Bitcoin bị nhiều người lo ngại rằng sẽ được dùng cho các giao dịch phạm pháp hoặc là rửa tiền. Nhưng quay lại với bản chất của Bitcoin một lần nữa, nó được sinh ra là để giải quyết bài toán ghi chép lại ai đã giao dịch với ai. Vì thế, mọi giao dịch đều được lưu lại và thống nhất ở nhiều nơi. Dù có thể không biết ai đứng đằng sau ví, mọi người đều có thể biết được giao dịch và phân tích khoanh vùng nếu họ thật sự muốn. Và vì thế, nếu muốn biết Bitcoin là tương lai nhân loại hay trò thổi bong bóng, hãy hỏi điều tương tự với mỗi hệ thống tài chính và tiền tệ từ mỗi quốc gia anh em đã và đang sinh sống câu hỏi tương tự mà anh em đã đặt cho Bitcoin:&lt;/p&gt;
+&lt;ul&gt;
+&lt;li&gt;Tiền đến từ đâu, tiền được tạo ra như thế nào?&lt;/li&gt;
+&lt;li&gt;Ai là người có quyền quyết định cung tiền? Ai là người kiểm soát cung tiền?&lt;/li&gt;
+&lt;li&gt;Giao dịch được ghi lại như thế nào?&lt;/li&gt;
+&lt;li&gt;Dòng tiền có minh bạch hay không, có sạch hay không?&lt;/li&gt;
+&lt;li&gt;Ở đâu bạn có 10 tỷ gửi tiết kiệm? &lt;/li&gt;
+&lt;li&gt;Từ đâu bạn có tiền mua biệt thự, mua Maybach, mua Porsche? &lt;/li&gt;
+&lt;li&gt;Nếu bạn làm mất địa chỉ ví cá nhân, bạn mất toàn bộ tài sản Bitcoin, vậy nếu như bạn đánh rơi ví tiền ở ngoài đường thì sao?&lt;/li&gt;
+&lt;/ul&gt;
 &lt;div class="footnote"&gt;
 &lt;hr /&gt;
 &lt;ol&gt;

</xml_diff>

<commit_message>
Mot so noi chua y tuong moi
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -1171,7 +1171,11 @@
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kinh tế</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
@@ -1185,10 +1189,14 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>- [ ] Nhân bản hoạt động - [ ]</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>data\blogs\Giá trị thặng dư.md</t>
@@ -1196,12 +1204,22 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t># Giá trị thặng dư</t>
+          <t># Giá trị thặng dư
+## 2 cách đạt được thặng dư
+## 
+- [ ] Nhân bản hoạt động
+- [ ]</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>&lt;h1 id="gia-tri-thang-du"&gt;Giá trị thặng dư&lt;/h1&gt;</t>
+          <t>&lt;h1 id="gia-tri-thang-du"&gt;Giá trị thặng dư&lt;/h1&gt;
+&lt;h2 id="2-cach-at-uoc-thang-du"&gt;2 cách đạt được thặng dư&lt;/h2&gt;
+&lt;h2 id="_1"&gt;&lt;/h2&gt;
+&lt;ul class="task-list"&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Nhân bản hoạt động&lt;/li&gt;
+&lt;li&gt;[ ]&lt;/li&gt;
+&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -2042,10 +2060,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tư duy</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>Quy Hai Ng</t>
@@ -2059,12 +2081,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>- [ ] Excel luôn là nơi - [ ] Hải vẫn đồng ý với quan điểm rằng chưa có phần mềm hay hệ thống nào có thể thay thế hoàn toàn Excel. - [ ] Nếu chúng hỗ trợ cho Excel</t>
+          <t>Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ `đổi mới`, `sáng tạo`, `start-up`. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo th...</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2074,30 +2096,70 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t># Một số nơi chứa ý tưởng mớ
+          <t># Một số nơi chứa ý tưởng mới
+Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ `đổi mới`, `sáng tạo`, `start-up`. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo thủ trong khi mọi thứ xung quanh đều đang thay đổi. Điều này không chỉ đúng với các cá nhân hay SME, mà còn đúng với cả các tập đoàn lớn.
+&gt; Innovation is everything! (Đổi mới là tất cả)
+&gt;
+&gt; -- &lt;cite&gt;Robert Noyce&lt;/cite&gt;
+Blog này sẽ không nói về những thời điểm bất chợt để hình thành ý tưởng mới như đi bộ, đi tắm, hay khi đi ngủ và nằm mơ,... Bài viết sẽ nói về những nơi có thể chứa nhiều ý tưởng mới. 
 ## Từ file excel
-- [ ] Excel luôn là nơi
-- [ ] Hải vẫn đồng ý với quan điểm rằng chưa có phần mềm hay hệ thống nào có thể thay thế hoàn toàn Excel.
-- [ ] Nếu chúng hỗ trợ cho Excel
+File excel luôn là nơi đọc và ghi lại thông tin theo thứ tự danh sách. Từ kế toán, thông tin quản lý nhân sự, tồn kho cho tới danh sách sản phẩm, bài viết. 
+Hải vẫn đồng ý với quan điểm rằng chưa một phần mềm kế toán hay quản lý nhân sự nào thực sự thay thế hoàn toàn Excel. Trước sau gì chúng cũng phải xuất ra Excel để theo dõi. Không cần biết phần mềm đó có mối quan hệ bảng và truy vấn phức tạp tới đâu. Và ngay cả khi tích hợp AI, các CRM hay ERP cũng không thoát khỏi việc nhập và xuất ra Excel. 
+Vậy những ý tưởng nào có thể ra đời từ Excel?
+- Ghi lại các ý tưởng và tổng hợp chúng vào Excel dưới bất kỳ template nào mà anh em mong muốn. [^1]
+- Tạo thống kê, biểu đồ trực quan, content từ file excel
+- Viết các script chuyển đổi, đọc ghi theo thời gian thực từ Excel
+Các báo cáo tài chính, các thống kê theo danh mục, các plan, và project management đều có thể chuyển qua chuyển lại về dạng excel theo cách này hoặc cách khác. Vì vậy ý tưởng có thể xuất hiện từ các excel template, excel list info và excel vba.
 ## Từ ứng dụng nhắn tin
-Về cơ bản, những gì bạn viết trên các ứng dụng nhắn tin sẽ định hình con người bạn như ngoài đời. 
+Với những phần mềm trao đổi công việc hay liên lạc, vẫn chưa có thứ gì có thể vượt qua được các ứng dụng nhắn tin mà chúng ta vẫn hay sử dụng hằng ngày. Và hầu hết chúng đều là miễn phí với những tính năng phổ thông và tính năng riêng biệt của từng app. Những lý do chính để các tin nhắn từ ứng dụng có thể là nơi chứa ý tưởng:
+- Đó là nơi định hình giao tiếp hằng ngày và mối quan hệ của một người, cũng là nơi ghi lại lịch sử cuộc trò chuyện. Nó vừa có tính riêng tư, vừa có tính lưu trữ. Và vì thế anh em có thể nhìn thấy vấn đề và tìm kiếm giải pháp từ chính đó.
+- Đó là nơi có sự đối thoại: hoặc là đối thoại 1-1, hoặc là đối thoại với nhóm. Nên ngoài là nơi hình thành ý tưởng, đó cũng có thể là nơi có những người để kiểm tra xem ý tưởng đó có khả thi hay không.
+- Với sự phát triển của AI ngày nay, chúng có thể can thiệp vào tin nhắn chat với chính mình, với nhóm để tóm tắt ý tưởng hoặc thực hiện triển khai các công việc cần thiết.
+OpenClaw về bản chất là kết nối Telegram với các ứng dụng để thực hiện các công việc hằng ngày. Từ thủ công, tự động cho tới lập trình, chúng đều có thể làm thông qua ứng dụng nhắn tin nếu anh em biết cấu hình và sử dụng AI.
+Nhược điểm của ứng dụng nhắn tin là nội dung tin nhắn có thể bị trôi bởi hơn 200 tin nhắn khác. Vì vậy, nếu ý tưởng anh em cho là ok, hãy ưu tiên ghi vào file ghi chú hoặc excel nhưng cũng nên nhắn với một người mà anh em thân và tin tưởng nhất nhất thay vì chỉ đơn giản là ghi vào đâu đó.
 ## Từ những cái cũ
-## Kết</t>
+Khác với việc tạo ra một thứ hoàn toàn mới, chúng ta hoàn toàn có thể tìm ý tưởng mới chỉ từ việc cải tiến những cái cũ. Về cơ bản thì thứ đó đã có sẵn nhưng vẫn có nhu cầu làm cho tốt hơn. Cũng là chiếc xe đó, nhưng nếu cải tiến động cơ làm cho tiết kiệm xăng hơn trước đây thì đó vẫn là ý tưởng mới vì chưa ai làm được. Tương tự là tối ưu hiệu năng phần mềm nhằm giảm tiêu thụ điện cũng như vùng nhớ chiếm dụng. Với cả dụng cụ cơ khí cũng vậy, nếu nó có thể nhỏ gọn hoặc gập gọn hơn những cái trước để tiện mang đi thì đó là sáng tạo. Không ai dám nói đó là ăn cắp bởi vì đơn giản chưa có ai làm chúng, đúng chứ? Các yếu tố có thể cải tiến (tùy vào tình huống) là: nhẹ hơn, bền hơn, tiết kiệm hơn, an toàn hơn, gọn hơn, nhanh hơn,... và rất nhiều chỉ số khác!
+[^1]: [Một cách kiếm tiền không mới nhưng luôn mới mẻ](https://haicogihay.com/blog/mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>&lt;h1 id="mot-so-noi-chua-y-tuong-mo"&gt;Một số nơi chứa ý tưởng mớ&lt;/h1&gt;
+          <t>&lt;h1 id="mot-so-noi-chua-y-tuong-moi"&gt;Một số nơi chứa ý tưởng mới&lt;/h1&gt;
+&lt;p&gt;Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ &lt;code&gt;đổi mới&lt;/code&gt;, &lt;code&gt;sáng tạo&lt;/code&gt;, &lt;code&gt;start-up&lt;/code&gt;. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo thủ trong khi mọi thứ xung quanh đều đang thay đổi. Điều này không chỉ đúng với các cá nhân hay SME, mà còn đúng với cả các tập đoàn lớn.&lt;/p&gt;
+&lt;blockquote&gt;
+&lt;p&gt;Innovation is everything! (Đổi mới là tất cả)&lt;/p&gt;
+&lt;p&gt;-- &lt;cite&gt;Robert Noyce&lt;/cite&gt;&lt;/p&gt;
+&lt;/blockquote&gt;
+&lt;p&gt;Blog này sẽ không nói về những thời điểm bất chợt để hình thành ý tưởng mới như đi bộ, đi tắm, hay khi đi ngủ và nằm mơ,... Bài viết sẽ nói về những nơi có thể chứa nhiều ý tưởng mới. &lt;/p&gt;
 &lt;h2 id="tu-file-excel"&gt;Từ file excel&lt;/h2&gt;
-&lt;ul class="task-list"&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Excel luôn là nơi&lt;/li&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Hải vẫn đồng ý với quan điểm rằng chưa có phần mềm hay hệ thống nào có thể thay thế hoàn toàn Excel.&lt;/li&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Nếu chúng hỗ trợ cho Excel&lt;/li&gt;
+&lt;p&gt;File excel luôn là nơi đọc và ghi lại thông tin theo thứ tự danh sách. Từ kế toán, thông tin quản lý nhân sự, tồn kho cho tới danh sách sản phẩm, bài viết. &lt;/p&gt;
+&lt;p&gt;Hải vẫn đồng ý với quan điểm rằng chưa một phần mềm kế toán hay quản lý nhân sự nào thực sự thay thế hoàn toàn Excel. Trước sau gì chúng cũng phải xuất ra Excel để theo dõi. Không cần biết phần mềm đó có mối quan hệ bảng và truy vấn phức tạp tới đâu. Và ngay cả khi tích hợp AI, các CRM hay ERP cũng không thoát khỏi việc nhập và xuất ra Excel. &lt;/p&gt;
+&lt;p&gt;Vậy những ý tưởng nào có thể ra đời từ Excel?&lt;/p&gt;
+&lt;ul&gt;
+&lt;li&gt;Ghi lại các ý tưởng và tổng hợp chúng vào Excel dưới bất kỳ template nào mà anh em mong muốn. &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt;&lt;/li&gt;
+&lt;li&gt;Tạo thống kê, biểu đồ trực quan, content từ file excel&lt;/li&gt;
+&lt;li&gt;Viết các script chuyển đổi, đọc ghi theo thời gian thực từ Excel&lt;/li&gt;
 &lt;/ul&gt;
+&lt;p&gt;Các báo cáo tài chính, các thống kê theo danh mục, các plan, và project management đều có thể chuyển qua chuyển lại về dạng excel theo cách này hoặc cách khác. Vì vậy ý tưởng có thể xuất hiện từ các excel template, excel list info và excel vba.&lt;/p&gt;
 &lt;h2 id="tu-ung-dung-nhan-tin"&gt;Từ ứng dụng nhắn tin&lt;/h2&gt;
-&lt;p&gt;Về cơ bản, những gì bạn viết trên các ứng dụng nhắn tin sẽ định hình con người bạn như ngoài đời. &lt;/p&gt;
+&lt;p&gt;Với những phần mềm trao đổi công việc hay liên lạc, vẫn chưa có thứ gì có thể vượt qua được các ứng dụng nhắn tin mà chúng ta vẫn hay sử dụng hằng ngày. Và hầu hết chúng đều là miễn phí với những tính năng phổ thông và tính năng riêng biệt của từng app. Những lý do chính để các tin nhắn từ ứng dụng có thể là nơi chứa ý tưởng:&lt;/p&gt;
+&lt;ul&gt;
+&lt;li&gt;Đó là nơi định hình giao tiếp hằng ngày và mối quan hệ của một người, cũng là nơi ghi lại lịch sử cuộc trò chuyện. Nó vừa có tính riêng tư, vừa có tính lưu trữ. Và vì thế anh em có thể nhìn thấy vấn đề và tìm kiếm giải pháp từ chính đó.&lt;/li&gt;
+&lt;li&gt;Đó là nơi có sự đối thoại: hoặc là đối thoại 1-1, hoặc là đối thoại với nhóm. Nên ngoài là nơi hình thành ý tưởng, đó cũng có thể là nơi có những người để kiểm tra xem ý tưởng đó có khả thi hay không.&lt;/li&gt;
+&lt;li&gt;Với sự phát triển của AI ngày nay, chúng có thể can thiệp vào tin nhắn chat với chính mình, với nhóm để tóm tắt ý tưởng hoặc thực hiện triển khai các công việc cần thiết.&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;OpenClaw về bản chất là kết nối Telegram với các ứng dụng để thực hiện các công việc hằng ngày. Từ thủ công, tự động cho tới lập trình, chúng đều có thể làm thông qua ứng dụng nhắn tin nếu anh em biết cấu hình và sử dụng AI.&lt;/p&gt;
+&lt;p&gt;Nhược điểm của ứng dụng nhắn tin là nội dung tin nhắn có thể bị trôi bởi hơn 200 tin nhắn khác. Vì vậy, nếu ý tưởng anh em cho là ok, hãy ưu tiên ghi vào file ghi chú hoặc excel nhưng cũng nên nhắn với một người mà anh em thân và tin tưởng nhất nhất thay vì chỉ đơn giản là ghi vào đâu đó.&lt;/p&gt;
 &lt;h2 id="tu-nhung-cai-cu"&gt;Từ những cái cũ&lt;/h2&gt;
-&lt;h2 id="ket"&gt;Kết&lt;/h2&gt;</t>
+&lt;p&gt;Khác với việc tạo ra một thứ hoàn toàn mới, chúng ta hoàn toàn có thể tìm ý tưởng mới chỉ từ việc cải tiến những cái cũ. Về cơ bản thì thứ đó đã có sẵn nhưng vẫn có nhu cầu làm cho tốt hơn. Cũng là chiếc xe đó, nhưng nếu cải tiến động cơ làm cho tiết kiệm xăng hơn trước đây thì đó vẫn là ý tưởng mới vì chưa ai làm được. Tương tự là tối ưu hiệu năng phần mềm nhằm giảm tiêu thụ điện cũng như vùng nhớ chiếm dụng. Với cả dụng cụ cơ khí cũng vậy, nếu nó có thể nhỏ gọn hoặc gập gọn hơn những cái trước để tiện mang đi thì đó là sáng tạo. Không ai dám nói đó là ăn cắp bởi vì đơn giản chưa có ai làm chúng, đúng chứ? Các yếu tố có thể cải tiến (tùy vào tình huống) là: nhẹ hơn, bền hơn, tiết kiệm hơn, an toàn hơn, gọn hơn, nhanh hơn,... và rất nhiều chỉ số khác!&lt;/p&gt;
+&lt;div class="footnote"&gt;
+&lt;hr /&gt;
+&lt;ol&gt;
+&lt;li id="fn:1"&gt;
+&lt;p&gt;&lt;a href="https://haicogihay.com/blog/mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me"&gt;Một cách kiếm tiền không mới nhưng luôn mới mẻ&lt;/a&gt;&amp;#160;&lt;a class="footnote-backref" href="#fnref:1" title="Jump back to footnote 1 in the text"&gt;&amp;#8617;&lt;/a&gt;&lt;/p&gt;
+&lt;/li&gt;
+&lt;/ol&gt;
+&lt;/div&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>